<commit_message>
docs: keluarkan fitur COD dari rancangan fitur
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HmiNd1QbTyjAfj7oGbYGxq
</commit_message>
<xml_diff>
--- a/docs/rancangan-fitur-marketplace-umkm.xlsx
+++ b/docs/rancangan-fitur-marketplace-umkm.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Roadmap" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Daftar Fitur'!$A$1:$K$101</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Daftar Fitur'!$A$1:$K$100</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="740" uniqueCount="419">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="415">
   <si>
     <t xml:space="preserve">Rancangan Fitur Marketplace UMKM — Gap Analysis Repository myumkm</t>
   </si>
@@ -381,18 +381,6 @@
     <t xml:space="preserve">Payment.php, libraries/Duitku.php</t>
   </si>
   <si>
-    <t xml:space="preserve">COD / bayar di tempat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Banyak pembeli daerah belum percaya bayar di muka</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Opsi COD dengan batas nominal per toko.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ada sisa logika cod di Payment.php, tetapi Checkout::place selalu memakai Duitku</t>
-  </si>
-  <si>
     <t xml:space="preserve">Voucher &amp; promo</t>
   </si>
   <si>
@@ -1269,7 +1257,7 @@
     <t xml:space="preserve">Pembeda utama (2–4 sprint)</t>
   </si>
   <si>
-    <t xml:space="preserve">pembukuan sederhana + laporan penjualan, pre-order fleksibel per produk (DP &amp; kalender), COD dengan batas nominal, pickup di toko.</t>
+    <t xml:space="preserve">pembukuan sederhana + laporan penjualan, pre-order fleksibel per produk (DP &amp; kalender), pickup di toko.</t>
   </si>
   <si>
     <t xml:space="preserve">Naik kelas (jangka menengah)</t>
@@ -1912,32 +1900,32 @@
         <v>10</v>
       </c>
       <c r="B5" s="5" t="n">
-        <f aca="false">COUNTIF('Daftar Fitur'!$B$2:$B$101,A5)</f>
-        <v>37</v>
+        <f aca="false">COUNTIF('Daftar Fitur'!$B$2:$B$100,A5)</f>
+        <v>36</v>
       </c>
       <c r="C5" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$101,A5,'Daftar Fitur'!$E$2:$E$101,"Ada")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A5,'Daftar Fitur'!$E$2:$E$100,"Ada")</f>
         <v>22</v>
       </c>
       <c r="D5" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$101,A5,'Daftar Fitur'!$E$2:$E$101,"Belum")</f>
-        <v>15</v>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A5,'Daftar Fitur'!$E$2:$E$100,"Belum")</f>
+        <v>14</v>
       </c>
       <c r="E5" s="6" t="n">
         <f aca="false">IF(B5=0,0,C5/B5)</f>
-        <v>0.594594594594595</v>
+        <v>0.611111111111111</v>
       </c>
       <c r="F5" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$101,A5,'Daftar Fitur'!$F$2:$F$101,"Ya")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A5,'Daftar Fitur'!$F$2:$F$100,"Ya")</f>
         <v>5</v>
       </c>
       <c r="G5" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$101,A5,'Daftar Fitur'!$F$2:$F$101,"Ya",'Daftar Fitur'!$E$2:$E$101,"Belum")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A5,'Daftar Fitur'!$F$2:$F$100,"Ya",'Daftar Fitur'!$E$2:$E$100,"Belum")</f>
         <v>4</v>
       </c>
       <c r="H5" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$101,A5,'Daftar Fitur'!$G$2:$G$101,"Ya")</f>
-        <v>9</v>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A5,'Daftar Fitur'!$G$2:$G$100,"Ya")</f>
+        <v>8</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1945,15 +1933,15 @@
         <v>11</v>
       </c>
       <c r="B6" s="5" t="n">
-        <f aca="false">COUNTIF('Daftar Fitur'!$B$2:$B$101,A6)</f>
+        <f aca="false">COUNTIF('Daftar Fitur'!$B$2:$B$100,A6)</f>
         <v>41</v>
       </c>
       <c r="C6" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$101,A6,'Daftar Fitur'!$E$2:$E$101,"Ada")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A6,'Daftar Fitur'!$E$2:$E$100,"Ada")</f>
         <v>21</v>
       </c>
       <c r="D6" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$101,A6,'Daftar Fitur'!$E$2:$E$101,"Belum")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A6,'Daftar Fitur'!$E$2:$E$100,"Belum")</f>
         <v>20</v>
       </c>
       <c r="E6" s="6" t="n">
@@ -1961,15 +1949,15 @@
         <v>0.51219512195122</v>
       </c>
       <c r="F6" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$101,A6,'Daftar Fitur'!$F$2:$F$101,"Ya")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A6,'Daftar Fitur'!$F$2:$F$100,"Ya")</f>
         <v>10</v>
       </c>
       <c r="G6" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$101,A6,'Daftar Fitur'!$F$2:$F$101,"Ya",'Daftar Fitur'!$E$2:$E$101,"Belum")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A6,'Daftar Fitur'!$F$2:$F$100,"Ya",'Daftar Fitur'!$E$2:$E$100,"Belum")</f>
         <v>8</v>
       </c>
       <c r="H6" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$101,A6,'Daftar Fitur'!$G$2:$G$101,"Ya")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A6,'Daftar Fitur'!$G$2:$G$100,"Ya")</f>
         <v>8</v>
       </c>
     </row>
@@ -1978,15 +1966,15 @@
         <v>12</v>
       </c>
       <c r="B7" s="5" t="n">
-        <f aca="false">COUNTIF('Daftar Fitur'!$B$2:$B$101,A7)</f>
+        <f aca="false">COUNTIF('Daftar Fitur'!$B$2:$B$100,A7)</f>
         <v>22</v>
       </c>
       <c r="C7" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$101,A7,'Daftar Fitur'!$E$2:$E$101,"Ada")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A7,'Daftar Fitur'!$E$2:$E$100,"Ada")</f>
         <v>9</v>
       </c>
       <c r="D7" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$101,A7,'Daftar Fitur'!$E$2:$E$101,"Belum")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A7,'Daftar Fitur'!$E$2:$E$100,"Belum")</f>
         <v>13</v>
       </c>
       <c r="E7" s="6" t="n">
@@ -1994,15 +1982,15 @@
         <v>0.409090909090909</v>
       </c>
       <c r="F7" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$101,A7,'Daftar Fitur'!$F$2:$F$101,"Ya")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A7,'Daftar Fitur'!$F$2:$F$100,"Ya")</f>
         <v>2</v>
       </c>
       <c r="G7" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$101,A7,'Daftar Fitur'!$F$2:$F$101,"Ya",'Daftar Fitur'!$E$2:$E$101,"Belum")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A7,'Daftar Fitur'!$F$2:$F$100,"Ya",'Daftar Fitur'!$E$2:$E$100,"Belum")</f>
         <v>2</v>
       </c>
       <c r="H7" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$101,A7,'Daftar Fitur'!$G$2:$G$101,"Ya")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A7,'Daftar Fitur'!$G$2:$G$100,"Ya")</f>
         <v>0</v>
       </c>
     </row>
@@ -2012,7 +2000,7 @@
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">SUM(B5:B7)</f>
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C8" s="8" t="n">
         <f aca="false">SUM(C5:C7)</f>
@@ -2020,11 +2008,11 @@
       </c>
       <c r="D8" s="8" t="n">
         <f aca="false">SUM(D5:D7)</f>
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E8" s="9" t="n">
         <f aca="false">IF(B8=0,0,C8/B8)</f>
-        <v>0.52</v>
+        <v>0.525252525252525</v>
       </c>
       <c r="F8" s="8" t="n">
         <f aca="false">SUM(F5:F7)</f>
@@ -2036,7 +2024,7 @@
       </c>
       <c r="H8" s="8" t="n">
         <f aca="false">SUM(H5:H7)</f>
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2108,7 +2096,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K101"/>
+  <dimension ref="A1:K100"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -2787,18 +2775,14 @@
         <v>17</v>
       </c>
       <c r="F23" s="13"/>
-      <c r="G23" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="G23" s="13"/>
       <c r="H23" s="14" t="s">
         <v>119</v>
       </c>
       <c r="I23" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="J23" s="14" t="s">
-        <v>121</v>
-      </c>
+      <c r="J23" s="14"/>
       <c r="K23" s="16"/>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2812,18 +2796,20 @@
         <v>101</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E24" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F24" s="13"/>
+      <c r="F24" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="G24" s="13"/>
       <c r="H24" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="I24" s="14" t="s">
         <v>123</v>
-      </c>
-      <c r="I24" s="14" t="s">
-        <v>124</v>
       </c>
       <c r="J24" s="14"/>
       <c r="K24" s="16"/>
@@ -2839,7 +2825,7 @@
         <v>101</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E25" s="13" t="s">
         <v>17</v>
@@ -2849,12 +2835,14 @@
       </c>
       <c r="G25" s="13"/>
       <c r="H25" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="I25" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="I25" s="14" t="s">
+      <c r="J25" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="J25" s="14"/>
       <c r="K25" s="16"/>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2883,12 +2871,10 @@
       <c r="I26" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="J26" s="14" t="s">
-        <v>131</v>
-      </c>
+      <c r="J26" s="14"/>
       <c r="K26" s="16"/>
     </row>
-    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="n">
         <v>26</v>
       </c>
@@ -2896,17 +2882,15 @@
         <v>10</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
       <c r="D27" s="15" t="s">
         <v>132</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F27" s="13" t="s">
-        <v>41</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="F27" s="13"/>
       <c r="G27" s="13"/>
       <c r="H27" s="14" t="s">
         <v>133</v>
@@ -2914,7 +2898,9 @@
       <c r="I27" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="J27" s="14"/>
+      <c r="J27" s="14" t="s">
+        <v>135</v>
+      </c>
       <c r="K27" s="16"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2925,7 +2911,7 @@
         <v>10</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D28" s="15" t="s">
         <v>136</v>
@@ -2954,7 +2940,7 @@
         <v>10</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D29" s="15" t="s">
         <v>140</v>
@@ -2983,7 +2969,7 @@
         <v>10</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D30" s="15" t="s">
         <v>144</v>
@@ -3012,7 +2998,7 @@
         <v>10</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D31" s="15" t="s">
         <v>148</v>
@@ -3033,7 +3019,7 @@
       </c>
       <c r="K31" s="16"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="n">
         <v>31</v>
       </c>
@@ -3041,7 +3027,7 @@
         <v>10</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D32" s="15" t="s">
         <v>152</v>
@@ -3062,7 +3048,7 @@
       </c>
       <c r="K32" s="16"/>
     </row>
-    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="n">
         <v>32</v>
       </c>
@@ -3070,7 +3056,7 @@
         <v>10</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D33" s="15" t="s">
         <v>156</v>
@@ -3099,28 +3085,28 @@
         <v>10</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D34" s="15" t="s">
         <v>160</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F34" s="13"/>
-      <c r="G34" s="13"/>
+      <c r="G34" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="H34" s="14" t="s">
         <v>161</v>
       </c>
       <c r="I34" s="14" t="s">
         <v>162</v>
       </c>
-      <c r="J34" s="14" t="s">
-        <v>163</v>
-      </c>
+      <c r="J34" s="14"/>
       <c r="K34" s="16"/>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="n">
         <v>34</v>
       </c>
@@ -3128,13 +3114,13 @@
         <v>10</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>135</v>
+        <v>163</v>
       </c>
       <c r="D35" s="15" t="s">
         <v>164</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F35" s="13"/>
       <c r="G35" s="13" t="s">
@@ -3146,7 +3132,9 @@
       <c r="I35" s="14" t="s">
         <v>166</v>
       </c>
-      <c r="J35" s="14"/>
+      <c r="J35" s="14" t="s">
+        <v>167</v>
+      </c>
       <c r="K35" s="16"/>
     </row>
     <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3157,13 +3145,13 @@
         <v>10</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D36" s="15" t="s">
         <v>168</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F36" s="13"/>
       <c r="G36" s="13" t="s">
@@ -3175,9 +3163,7 @@
       <c r="I36" s="14" t="s">
         <v>170</v>
       </c>
-      <c r="J36" s="14" t="s">
-        <v>171</v>
-      </c>
+      <c r="J36" s="14"/>
       <c r="K36" s="16"/>
     </row>
     <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3188,10 +3174,10 @@
         <v>10</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E37" s="13" t="s">
         <v>17</v>
@@ -3201,10 +3187,10 @@
         <v>41</v>
       </c>
       <c r="H37" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="I37" s="14" t="s">
         <v>173</v>
-      </c>
-      <c r="I37" s="14" t="s">
-        <v>174</v>
       </c>
       <c r="J37" s="14"/>
       <c r="K37" s="16"/>
@@ -3214,16 +3200,16 @@
         <v>37</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="D38" s="15" t="s">
         <v>175</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F38" s="13"/>
       <c r="G38" s="13" t="s">
@@ -3235,7 +3221,9 @@
       <c r="I38" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="J38" s="14"/>
+      <c r="J38" s="14" t="s">
+        <v>178</v>
+      </c>
       <c r="K38" s="16"/>
     </row>
     <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3246,7 +3234,7 @@
         <v>11</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D39" s="15" t="s">
         <v>179</v>
@@ -3255,9 +3243,7 @@
         <v>15</v>
       </c>
       <c r="F39" s="13"/>
-      <c r="G39" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="G39" s="13"/>
       <c r="H39" s="14" t="s">
         <v>180</v>
       </c>
@@ -3277,7 +3263,7 @@
         <v>11</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D40" s="15" t="s">
         <v>183</v>
@@ -3306,25 +3292,25 @@
         <v>11</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D41" s="15" t="s">
         <v>187</v>
       </c>
       <c r="E41" s="13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F41" s="13"/>
-      <c r="G41" s="13"/>
+      <c r="G41" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="H41" s="14" t="s">
         <v>188</v>
       </c>
       <c r="I41" s="14" t="s">
         <v>189</v>
       </c>
-      <c r="J41" s="14" t="s">
-        <v>190</v>
-      </c>
+      <c r="J41" s="14"/>
       <c r="K41" s="16"/>
     </row>
     <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3335,23 +3321,23 @@
         <v>11</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D42" s="15" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E42" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F42" s="13"/>
-      <c r="G42" s="13" t="s">
+      <c r="F42" s="13" t="s">
         <v>41</v>
       </c>
+      <c r="G42" s="13"/>
       <c r="H42" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="I42" s="14" t="s">
         <v>192</v>
-      </c>
-      <c r="I42" s="14" t="s">
-        <v>193</v>
       </c>
       <c r="J42" s="14"/>
       <c r="K42" s="16"/>
@@ -3364,25 +3350,25 @@
         <v>11</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D43" s="15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E43" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F43" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="F43" s="13"/>
       <c r="G43" s="13"/>
       <c r="H43" s="14" t="s">
+        <v>194</v>
+      </c>
+      <c r="I43" s="14" t="s">
         <v>195</v>
       </c>
-      <c r="I43" s="14" t="s">
+      <c r="J43" s="14" t="s">
         <v>196</v>
       </c>
-      <c r="J43" s="14"/>
       <c r="K43" s="16"/>
     </row>
     <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3393,24 +3379,24 @@
         <v>11</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>178</v>
+        <v>197</v>
       </c>
       <c r="D44" s="15" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F44" s="13"/>
       <c r="G44" s="13"/>
       <c r="H44" s="14" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I44" s="14" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="J44" s="14" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="K44" s="16"/>
     </row>
@@ -3422,7 +3408,7 @@
         <v>11</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="D45" s="15" t="s">
         <v>202</v>
@@ -3451,7 +3437,7 @@
         <v>11</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="D46" s="15" t="s">
         <v>206</v>
@@ -3480,7 +3466,7 @@
         <v>11</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="D47" s="15" t="s">
         <v>210</v>
@@ -3509,7 +3495,7 @@
         <v>11</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="D48" s="15" t="s">
         <v>214</v>
@@ -3517,8 +3503,12 @@
       <c r="E48" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="F48" s="13"/>
-      <c r="G48" s="13"/>
+      <c r="F48" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="G48" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="H48" s="14" t="s">
         <v>215</v>
       </c>
@@ -3538,7 +3528,7 @@
         <v>11</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="D49" s="15" t="s">
         <v>218</v>
@@ -3546,12 +3536,8 @@
       <c r="E49" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="F49" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="G49" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="F49" s="13"/>
+      <c r="G49" s="13"/>
       <c r="H49" s="14" t="s">
         <v>219</v>
       </c>
@@ -3571,25 +3557,25 @@
         <v>11</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="D50" s="15" t="s">
         <v>222</v>
       </c>
       <c r="E50" s="13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F50" s="13"/>
-      <c r="G50" s="13"/>
+      <c r="G50" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="H50" s="14" t="s">
         <v>223</v>
       </c>
       <c r="I50" s="14" t="s">
         <v>224</v>
       </c>
-      <c r="J50" s="14" t="s">
-        <v>225</v>
-      </c>
+      <c r="J50" s="14"/>
       <c r="K50" s="16"/>
     </row>
     <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3600,23 +3586,21 @@
         <v>11</v>
       </c>
       <c r="C51" s="14" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="D51" s="15" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E51" s="13" t="s">
         <v>17</v>
       </c>
       <c r="F51" s="13"/>
-      <c r="G51" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="G51" s="13"/>
       <c r="H51" s="14" t="s">
+        <v>226</v>
+      </c>
+      <c r="I51" s="14" t="s">
         <v>227</v>
-      </c>
-      <c r="I51" s="14" t="s">
-        <v>228</v>
       </c>
       <c r="J51" s="14"/>
       <c r="K51" s="16"/>
@@ -3629,10 +3613,10 @@
         <v>11</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="D52" s="15" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E52" s="13" t="s">
         <v>17</v>
@@ -3640,10 +3624,10 @@
       <c r="F52" s="13"/>
       <c r="G52" s="13"/>
       <c r="H52" s="14" t="s">
+        <v>229</v>
+      </c>
+      <c r="I52" s="14" t="s">
         <v>230</v>
-      </c>
-      <c r="I52" s="14" t="s">
-        <v>231</v>
       </c>
       <c r="J52" s="14"/>
       <c r="K52" s="16"/>
@@ -3656,21 +3640,23 @@
         <v>11</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="D53" s="15" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E53" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F53" s="13"/>
+      <c r="F53" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="G53" s="13"/>
       <c r="H53" s="14" t="s">
+        <v>232</v>
+      </c>
+      <c r="I53" s="14" t="s">
         <v>233</v>
-      </c>
-      <c r="I53" s="14" t="s">
-        <v>234</v>
       </c>
       <c r="J53" s="14"/>
       <c r="K53" s="16"/>
@@ -3683,10 +3669,10 @@
         <v>11</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="D54" s="15" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E54" s="13" t="s">
         <v>17</v>
@@ -3696,10 +3682,10 @@
       </c>
       <c r="G54" s="13"/>
       <c r="H54" s="14" t="s">
+        <v>235</v>
+      </c>
+      <c r="I54" s="14" t="s">
         <v>236</v>
-      </c>
-      <c r="I54" s="14" t="s">
-        <v>237</v>
       </c>
       <c r="J54" s="14"/>
       <c r="K54" s="16"/>
@@ -3712,25 +3698,27 @@
         <v>11</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>201</v>
+        <v>237</v>
       </c>
       <c r="D55" s="15" t="s">
         <v>238</v>
       </c>
       <c r="E55" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F55" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F55" s="13"/>
+      <c r="G55" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="G55" s="13"/>
       <c r="H55" s="14" t="s">
         <v>239</v>
       </c>
       <c r="I55" s="14" t="s">
         <v>240</v>
       </c>
-      <c r="J55" s="14"/>
+      <c r="J55" s="14" t="s">
+        <v>241</v>
+      </c>
       <c r="K55" s="16"/>
     </row>
     <row r="56" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3741,7 +3729,7 @@
         <v>11</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="D56" s="15" t="s">
         <v>242</v>
@@ -3750,9 +3738,7 @@
         <v>15</v>
       </c>
       <c r="F56" s="13"/>
-      <c r="G56" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="G56" s="13"/>
       <c r="H56" s="14" t="s">
         <v>243</v>
       </c>
@@ -3772,7 +3758,7 @@
         <v>11</v>
       </c>
       <c r="C57" s="14" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="D57" s="15" t="s">
         <v>246</v>
@@ -3780,7 +3766,9 @@
       <c r="E57" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="F57" s="13"/>
+      <c r="F57" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="G57" s="13"/>
       <c r="H57" s="14" t="s">
         <v>247</v>
@@ -3801,7 +3789,7 @@
         <v>11</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="D58" s="15" t="s">
         <v>250</v>
@@ -3809,9 +3797,7 @@
       <c r="E58" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="F58" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="F58" s="13"/>
       <c r="G58" s="13"/>
       <c r="H58" s="14" t="s">
         <v>251</v>
@@ -3832,7 +3818,7 @@
         <v>11</v>
       </c>
       <c r="C59" s="14" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="D59" s="15" t="s">
         <v>254</v>
@@ -3861,7 +3847,7 @@
         <v>11</v>
       </c>
       <c r="C60" s="14" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="D60" s="15" t="s">
         <v>258</v>
@@ -3890,7 +3876,7 @@
         <v>11</v>
       </c>
       <c r="C61" s="14" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="D61" s="15" t="s">
         <v>262</v>
@@ -3919,7 +3905,7 @@
         <v>11</v>
       </c>
       <c r="C62" s="14" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="D62" s="15" t="s">
         <v>266</v>
@@ -3948,13 +3934,13 @@
         <v>11</v>
       </c>
       <c r="C63" s="14" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="D63" s="15" t="s">
         <v>270</v>
       </c>
       <c r="E63" s="13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F63" s="13"/>
       <c r="G63" s="13"/>
@@ -3964,9 +3950,7 @@
       <c r="I63" s="14" t="s">
         <v>272</v>
       </c>
-      <c r="J63" s="14" t="s">
-        <v>273</v>
-      </c>
+      <c r="J63" s="14"/>
       <c r="K63" s="16"/>
     </row>
     <row r="64" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3977,21 +3961,23 @@
         <v>11</v>
       </c>
       <c r="C64" s="14" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="D64" s="15" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E64" s="13" t="s">
         <v>17</v>
       </c>
       <c r="F64" s="13"/>
-      <c r="G64" s="13"/>
+      <c r="G64" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="H64" s="14" t="s">
+        <v>274</v>
+      </c>
+      <c r="I64" s="14" t="s">
         <v>275</v>
-      </c>
-      <c r="I64" s="14" t="s">
-        <v>276</v>
       </c>
       <c r="J64" s="14"/>
       <c r="K64" s="16"/>
@@ -4004,23 +3990,21 @@
         <v>11</v>
       </c>
       <c r="C65" s="14" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="D65" s="15" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E65" s="13" t="s">
         <v>17</v>
       </c>
       <c r="F65" s="13"/>
-      <c r="G65" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="G65" s="13"/>
       <c r="H65" s="14" t="s">
+        <v>277</v>
+      </c>
+      <c r="I65" s="14" t="s">
         <v>278</v>
-      </c>
-      <c r="I65" s="14" t="s">
-        <v>279</v>
       </c>
       <c r="J65" s="14"/>
       <c r="K65" s="16"/>
@@ -4033,13 +4017,13 @@
         <v>11</v>
       </c>
       <c r="C66" s="14" t="s">
-        <v>241</v>
+        <v>279</v>
       </c>
       <c r="D66" s="15" t="s">
         <v>280</v>
       </c>
       <c r="E66" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F66" s="13"/>
       <c r="G66" s="13"/>
@@ -4049,7 +4033,9 @@
       <c r="I66" s="14" t="s">
         <v>282</v>
       </c>
-      <c r="J66" s="14"/>
+      <c r="J66" s="14" t="s">
+        <v>283</v>
+      </c>
       <c r="K66" s="16"/>
     </row>
     <row r="67" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4060,7 +4046,7 @@
         <v>11</v>
       </c>
       <c r="C67" s="14" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="D67" s="15" t="s">
         <v>284</v>
@@ -4089,7 +4075,7 @@
         <v>11</v>
       </c>
       <c r="C68" s="14" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="D68" s="15" t="s">
         <v>288</v>
@@ -4118,25 +4104,25 @@
         <v>11</v>
       </c>
       <c r="C69" s="14" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="D69" s="15" t="s">
         <v>292</v>
       </c>
       <c r="E69" s="13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F69" s="13"/>
-      <c r="G69" s="13"/>
+      <c r="G69" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="H69" s="14" t="s">
         <v>293</v>
       </c>
       <c r="I69" s="14" t="s">
         <v>294</v>
       </c>
-      <c r="J69" s="14" t="s">
-        <v>295</v>
-      </c>
+      <c r="J69" s="14"/>
       <c r="K69" s="16"/>
     </row>
     <row r="70" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4147,28 +4133,28 @@
         <v>11</v>
       </c>
       <c r="C70" s="14" t="s">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="D70" s="15" t="s">
         <v>296</v>
       </c>
       <c r="E70" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F70" s="13"/>
-      <c r="G70" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="G70" s="13"/>
       <c r="H70" s="14" t="s">
         <v>297</v>
       </c>
       <c r="I70" s="14" t="s">
         <v>298</v>
       </c>
-      <c r="J70" s="14"/>
+      <c r="J70" s="14" t="s">
+        <v>299</v>
+      </c>
       <c r="K70" s="16"/>
     </row>
-    <row r="71" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="13" t="n">
         <v>70</v>
       </c>
@@ -4176,28 +4162,30 @@
         <v>11</v>
       </c>
       <c r="C71" s="14" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="D71" s="15" t="s">
         <v>300</v>
       </c>
       <c r="E71" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F71" s="13"/>
-      <c r="G71" s="13"/>
+        <v>17</v>
+      </c>
+      <c r="F71" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="G71" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="H71" s="14" t="s">
         <v>301</v>
       </c>
       <c r="I71" s="14" t="s">
         <v>302</v>
       </c>
-      <c r="J71" s="14" t="s">
-        <v>303</v>
-      </c>
+      <c r="J71" s="14"/>
       <c r="K71" s="16"/>
     </row>
-    <row r="72" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="13" t="n">
         <v>71</v>
       </c>
@@ -4205,10 +4193,10 @@
         <v>11</v>
       </c>
       <c r="C72" s="14" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="D72" s="15" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="E72" s="13" t="s">
         <v>17</v>
@@ -4216,14 +4204,12 @@
       <c r="F72" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="G72" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="G72" s="13"/>
       <c r="H72" s="14" t="s">
+        <v>304</v>
+      </c>
+      <c r="I72" s="14" t="s">
         <v>305</v>
-      </c>
-      <c r="I72" s="14" t="s">
-        <v>306</v>
       </c>
       <c r="J72" s="14"/>
       <c r="K72" s="16"/>
@@ -4236,23 +4222,21 @@
         <v>11</v>
       </c>
       <c r="C73" s="14" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="D73" s="15" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="E73" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F73" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="F73" s="13"/>
       <c r="G73" s="13"/>
       <c r="H73" s="14" t="s">
+        <v>307</v>
+      </c>
+      <c r="I73" s="14" t="s">
         <v>308</v>
-      </c>
-      <c r="I73" s="14" t="s">
-        <v>309</v>
       </c>
       <c r="J73" s="14"/>
       <c r="K73" s="16"/>
@@ -4265,21 +4249,23 @@
         <v>11</v>
       </c>
       <c r="C74" s="14" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="D74" s="15" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E74" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F74" s="13"/>
+      <c r="F74" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="G74" s="13"/>
       <c r="H74" s="14" t="s">
+        <v>310</v>
+      </c>
+      <c r="I74" s="14" t="s">
         <v>311</v>
-      </c>
-      <c r="I74" s="14" t="s">
-        <v>312</v>
       </c>
       <c r="J74" s="14"/>
       <c r="K74" s="16"/>
@@ -4292,23 +4278,21 @@
         <v>11</v>
       </c>
       <c r="C75" s="14" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="D75" s="15" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E75" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F75" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="F75" s="13"/>
       <c r="G75" s="13"/>
       <c r="H75" s="14" t="s">
+        <v>313</v>
+      </c>
+      <c r="I75" s="14" t="s">
         <v>314</v>
-      </c>
-      <c r="I75" s="14" t="s">
-        <v>315</v>
       </c>
       <c r="J75" s="14"/>
       <c r="K75" s="16"/>
@@ -4321,26 +4305,28 @@
         <v>11</v>
       </c>
       <c r="C76" s="14" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="D76" s="15" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E76" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F76" s="13"/>
+      <c r="F76" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="G76" s="13"/>
       <c r="H76" s="14" t="s">
+        <v>316</v>
+      </c>
+      <c r="I76" s="14" t="s">
         <v>317</v>
-      </c>
-      <c r="I76" s="14" t="s">
-        <v>318</v>
       </c>
       <c r="J76" s="14"/>
       <c r="K76" s="16"/>
     </row>
-    <row r="77" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="13" t="n">
         <v>76</v>
       </c>
@@ -4348,10 +4334,10 @@
         <v>11</v>
       </c>
       <c r="C77" s="14" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="D77" s="15" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E77" s="13" t="s">
         <v>17</v>
@@ -4361,15 +4347,15 @@
       </c>
       <c r="G77" s="13"/>
       <c r="H77" s="14" t="s">
+        <v>319</v>
+      </c>
+      <c r="I77" s="14" t="s">
         <v>320</v>
-      </c>
-      <c r="I77" s="14" t="s">
-        <v>321</v>
       </c>
       <c r="J77" s="14"/>
       <c r="K77" s="16"/>
     </row>
-    <row r="78" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="13" t="n">
         <v>77</v>
       </c>
@@ -4377,23 +4363,21 @@
         <v>11</v>
       </c>
       <c r="C78" s="14" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="D78" s="15" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="E78" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F78" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="F78" s="13"/>
       <c r="G78" s="13"/>
       <c r="H78" s="14" t="s">
+        <v>322</v>
+      </c>
+      <c r="I78" s="14" t="s">
         <v>323</v>
-      </c>
-      <c r="I78" s="14" t="s">
-        <v>324</v>
       </c>
       <c r="J78" s="14"/>
       <c r="K78" s="16"/>
@@ -4403,16 +4387,16 @@
         <v>78</v>
       </c>
       <c r="B79" s="14" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C79" s="14" t="s">
-        <v>299</v>
+        <v>324</v>
       </c>
       <c r="D79" s="15" t="s">
         <v>325</v>
       </c>
       <c r="E79" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F79" s="13"/>
       <c r="G79" s="13"/>
@@ -4422,7 +4406,9 @@
       <c r="I79" s="14" t="s">
         <v>327</v>
       </c>
-      <c r="J79" s="14"/>
+      <c r="J79" s="14" t="s">
+        <v>328</v>
+      </c>
       <c r="K79" s="16"/>
     </row>
     <row r="80" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4433,13 +4419,13 @@
         <v>12</v>
       </c>
       <c r="C80" s="14" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D80" s="15" t="s">
         <v>329</v>
       </c>
       <c r="E80" s="13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F80" s="13"/>
       <c r="G80" s="13"/>
@@ -4449,9 +4435,7 @@
       <c r="I80" s="14" t="s">
         <v>331</v>
       </c>
-      <c r="J80" s="14" t="s">
-        <v>332</v>
-      </c>
+      <c r="J80" s="14"/>
       <c r="K80" s="16"/>
     </row>
     <row r="81" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4462,21 +4446,23 @@
         <v>12</v>
       </c>
       <c r="C81" s="14" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D81" s="15" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="E81" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F81" s="13"/>
+      <c r="F81" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="G81" s="13"/>
       <c r="H81" s="14" t="s">
+        <v>333</v>
+      </c>
+      <c r="I81" s="14" t="s">
         <v>334</v>
-      </c>
-      <c r="I81" s="14" t="s">
-        <v>335</v>
       </c>
       <c r="J81" s="14"/>
       <c r="K81" s="16"/>
@@ -4489,17 +4475,15 @@
         <v>12</v>
       </c>
       <c r="C82" s="14" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
       <c r="D82" s="15" t="s">
         <v>336</v>
       </c>
       <c r="E82" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F82" s="13" t="s">
-        <v>41</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="F82" s="13"/>
       <c r="G82" s="13"/>
       <c r="H82" s="14" t="s">
         <v>337</v>
@@ -4507,7 +4491,9 @@
       <c r="I82" s="14" t="s">
         <v>338</v>
       </c>
-      <c r="J82" s="14"/>
+      <c r="J82" s="14" t="s">
+        <v>339</v>
+      </c>
       <c r="K82" s="16"/>
     </row>
     <row r="83" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4518,7 +4504,7 @@
         <v>12</v>
       </c>
       <c r="C83" s="14" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="D83" s="15" t="s">
         <v>340</v>
@@ -4547,13 +4533,13 @@
         <v>12</v>
       </c>
       <c r="C84" s="14" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="D84" s="15" t="s">
         <v>344</v>
       </c>
       <c r="E84" s="13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F84" s="13"/>
       <c r="G84" s="13"/>
@@ -4563,9 +4549,7 @@
       <c r="I84" s="14" t="s">
         <v>346</v>
       </c>
-      <c r="J84" s="14" t="s">
-        <v>347</v>
-      </c>
+      <c r="J84" s="14"/>
       <c r="K84" s="16"/>
     </row>
     <row r="85" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4576,21 +4560,23 @@
         <v>12</v>
       </c>
       <c r="C85" s="14" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="D85" s="15" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E85" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F85" s="13"/>
+      <c r="F85" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="G85" s="13"/>
       <c r="H85" s="14" t="s">
+        <v>348</v>
+      </c>
+      <c r="I85" s="14" t="s">
         <v>349</v>
-      </c>
-      <c r="I85" s="14" t="s">
-        <v>350</v>
       </c>
       <c r="J85" s="14"/>
       <c r="K85" s="16"/>
@@ -4603,17 +4589,15 @@
         <v>12</v>
       </c>
       <c r="C86" s="14" t="s">
-        <v>339</v>
+        <v>350</v>
       </c>
       <c r="D86" s="15" t="s">
         <v>351</v>
       </c>
       <c r="E86" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F86" s="13" t="s">
-        <v>41</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="F86" s="13"/>
       <c r="G86" s="13"/>
       <c r="H86" s="14" t="s">
         <v>352</v>
@@ -4621,7 +4605,9 @@
       <c r="I86" s="14" t="s">
         <v>353</v>
       </c>
-      <c r="J86" s="14"/>
+      <c r="J86" s="14" t="s">
+        <v>354</v>
+      </c>
       <c r="K86" s="16"/>
     </row>
     <row r="87" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4632,13 +4618,13 @@
         <v>12</v>
       </c>
       <c r="C87" s="14" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="D87" s="15" t="s">
         <v>355</v>
       </c>
       <c r="E87" s="13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F87" s="13"/>
       <c r="G87" s="13"/>
@@ -4648,9 +4634,7 @@
       <c r="I87" s="14" t="s">
         <v>357</v>
       </c>
-      <c r="J87" s="14" t="s">
-        <v>358</v>
-      </c>
+      <c r="J87" s="14"/>
       <c r="K87" s="16"/>
     </row>
     <row r="88" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4661,10 +4645,10 @@
         <v>12</v>
       </c>
       <c r="C88" s="14" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="D88" s="15" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E88" s="13" t="s">
         <v>17</v>
@@ -4672,10 +4656,10 @@
       <c r="F88" s="13"/>
       <c r="G88" s="13"/>
       <c r="H88" s="14" t="s">
+        <v>359</v>
+      </c>
+      <c r="I88" s="14" t="s">
         <v>360</v>
-      </c>
-      <c r="I88" s="14" t="s">
-        <v>361</v>
       </c>
       <c r="J88" s="14"/>
       <c r="K88" s="16"/>
@@ -4688,10 +4672,10 @@
         <v>12</v>
       </c>
       <c r="C89" s="14" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="D89" s="15" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E89" s="13" t="s">
         <v>17</v>
@@ -4699,10 +4683,10 @@
       <c r="F89" s="13"/>
       <c r="G89" s="13"/>
       <c r="H89" s="14" t="s">
+        <v>362</v>
+      </c>
+      <c r="I89" s="14" t="s">
         <v>363</v>
-      </c>
-      <c r="I89" s="14" t="s">
-        <v>364</v>
       </c>
       <c r="J89" s="14"/>
       <c r="K89" s="16"/>
@@ -4715,10 +4699,10 @@
         <v>12</v>
       </c>
       <c r="C90" s="14" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="D90" s="15" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E90" s="13" t="s">
         <v>17</v>
@@ -4726,10 +4710,10 @@
       <c r="F90" s="13"/>
       <c r="G90" s="13"/>
       <c r="H90" s="14" t="s">
+        <v>365</v>
+      </c>
+      <c r="I90" s="14" t="s">
         <v>366</v>
-      </c>
-      <c r="I90" s="14" t="s">
-        <v>367</v>
       </c>
       <c r="J90" s="14"/>
       <c r="K90" s="16"/>
@@ -4742,13 +4726,13 @@
         <v>12</v>
       </c>
       <c r="C91" s="14" t="s">
-        <v>354</v>
+        <v>367</v>
       </c>
       <c r="D91" s="15" t="s">
         <v>368</v>
       </c>
       <c r="E91" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F91" s="13"/>
       <c r="G91" s="13"/>
@@ -4758,7 +4742,9 @@
       <c r="I91" s="14" t="s">
         <v>370</v>
       </c>
-      <c r="J91" s="14"/>
+      <c r="J91" s="14" t="s">
+        <v>371</v>
+      </c>
       <c r="K91" s="16"/>
     </row>
     <row r="92" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4769,7 +4755,7 @@
         <v>12</v>
       </c>
       <c r="C92" s="14" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="D92" s="15" t="s">
         <v>372</v>
@@ -4798,7 +4784,7 @@
         <v>12</v>
       </c>
       <c r="C93" s="14" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="D93" s="15" t="s">
         <v>376</v>
@@ -4827,7 +4813,7 @@
         <v>12</v>
       </c>
       <c r="C94" s="14" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="D94" s="15" t="s">
         <v>380</v>
@@ -4856,13 +4842,13 @@
         <v>12</v>
       </c>
       <c r="C95" s="14" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="D95" s="15" t="s">
         <v>384</v>
       </c>
       <c r="E95" s="13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F95" s="13"/>
       <c r="G95" s="13"/>
@@ -4872,9 +4858,7 @@
       <c r="I95" s="14" t="s">
         <v>386</v>
       </c>
-      <c r="J95" s="14" t="s">
-        <v>387</v>
-      </c>
+      <c r="J95" s="14"/>
       <c r="K95" s="16"/>
     </row>
     <row r="96" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4885,10 +4869,10 @@
         <v>12</v>
       </c>
       <c r="C96" s="14" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="D96" s="15" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E96" s="13" t="s">
         <v>17</v>
@@ -4896,10 +4880,10 @@
       <c r="F96" s="13"/>
       <c r="G96" s="13"/>
       <c r="H96" s="14" t="s">
+        <v>388</v>
+      </c>
+      <c r="I96" s="14" t="s">
         <v>389</v>
-      </c>
-      <c r="I96" s="14" t="s">
-        <v>390</v>
       </c>
       <c r="J96" s="14"/>
       <c r="K96" s="16"/>
@@ -4912,10 +4896,10 @@
         <v>12</v>
       </c>
       <c r="C97" s="14" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="D97" s="15" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E97" s="13" t="s">
         <v>17</v>
@@ -4923,10 +4907,10 @@
       <c r="F97" s="13"/>
       <c r="G97" s="13"/>
       <c r="H97" s="14" t="s">
+        <v>391</v>
+      </c>
+      <c r="I97" s="14" t="s">
         <v>392</v>
-      </c>
-      <c r="I97" s="14" t="s">
-        <v>393</v>
       </c>
       <c r="J97" s="14"/>
       <c r="K97" s="16"/>
@@ -4939,7 +4923,7 @@
         <v>12</v>
       </c>
       <c r="C98" s="14" t="s">
-        <v>371</v>
+        <v>393</v>
       </c>
       <c r="D98" s="15" t="s">
         <v>394</v>
@@ -4966,10 +4950,10 @@
         <v>12</v>
       </c>
       <c r="C99" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="D99" s="15" t="s">
         <v>397</v>
-      </c>
-      <c r="D99" s="15" t="s">
-        <v>398</v>
       </c>
       <c r="E99" s="13" t="s">
         <v>17</v>
@@ -4977,12 +4961,14 @@
       <c r="F99" s="13"/>
       <c r="G99" s="13"/>
       <c r="H99" s="14" t="s">
+        <v>398</v>
+      </c>
+      <c r="I99" s="14" t="s">
         <v>399</v>
       </c>
-      <c r="I99" s="14" t="s">
+      <c r="J99" s="14" t="s">
         <v>400</v>
       </c>
-      <c r="J99" s="14"/>
       <c r="K99" s="16"/>
     </row>
     <row r="100" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4993,13 +4979,13 @@
         <v>12</v>
       </c>
       <c r="C100" s="14" t="s">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="D100" s="15" t="s">
         <v>401</v>
       </c>
       <c r="E100" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F100" s="13"/>
       <c r="G100" s="13"/>
@@ -5014,38 +5000,9 @@
       </c>
       <c r="K100" s="16"/>
     </row>
-    <row r="101" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="13" t="n">
-        <v>100</v>
-      </c>
-      <c r="B101" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="C101" s="14" t="s">
-        <v>397</v>
-      </c>
-      <c r="D101" s="15" t="s">
-        <v>405</v>
-      </c>
-      <c r="E101" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F101" s="13"/>
-      <c r="G101" s="13"/>
-      <c r="H101" s="14" t="s">
-        <v>406</v>
-      </c>
-      <c r="I101" s="14" t="s">
-        <v>407</v>
-      </c>
-      <c r="J101" s="14" t="s">
-        <v>408</v>
-      </c>
-      <c r="K101" s="16"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K101"/>
-  <conditionalFormatting sqref="E2:E101">
+  <autoFilter ref="A1:K100"/>
+  <conditionalFormatting sqref="E2:E100">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Ada"</formula>
     </cfRule>
@@ -5054,11 +5011,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E101" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E100" type="list">
       <formula1>"Ada,Belum,Sebagian"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K2:K101" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K2:K100" type="list">
       <formula1>"P1 - Quick win,P2 - Pembeda,P3 - Naik kelas,P4 - Skala"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -5088,42 +5045,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
-        <v>413</v>
+        <v>409</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>417</v>
+        <v>413</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: keluarkan fitur ambil sendiri di toko (pickup) dari rancangan fitur
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HmiNd1QbTyjAfj7oGbYGxq
</commit_message>
<xml_diff>
--- a/docs/rancangan-fitur-marketplace-umkm.xlsx
+++ b/docs/rancangan-fitur-marketplace-umkm.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Roadmap" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Daftar Fitur'!$A$1:$K$100</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Daftar Fitur'!$A$1:$K$99</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="412">
   <si>
     <t xml:space="preserve">Rancangan Fitur Marketplace UMKM — Gap Analysis Repository myumkm</t>
   </si>
@@ -411,15 +411,6 @@
     <t xml:space="preserve">Repo baru punya waktu_proses_hari di level toko</t>
   </si>
   <si>
-    <t xml:space="preserve">Ambil sendiri di toko (pickup)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tetangga satu kecamatan lebih suka mengambil sendiri</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Opsi ongkir 0 + jam ambil.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Pasca-Pembelian</t>
   </si>
   <si>
@@ -1257,7 +1248,7 @@
     <t xml:space="preserve">Pembeda utama (2–4 sprint)</t>
   </si>
   <si>
-    <t xml:space="preserve">pembukuan sederhana + laporan penjualan, pre-order fleksibel per produk (DP &amp; kalender), pickup di toko.</t>
+    <t xml:space="preserve">pembukuan sederhana + laporan penjualan, pre-order fleksibel per produk (DP &amp; kalender).</t>
   </si>
   <si>
     <t xml:space="preserve">Naik kelas (jangka menengah)</t>
@@ -1900,31 +1891,31 @@
         <v>10</v>
       </c>
       <c r="B5" s="5" t="n">
-        <f aca="false">COUNTIF('Daftar Fitur'!$B$2:$B$100,A5)</f>
-        <v>36</v>
+        <f aca="false">COUNTIF('Daftar Fitur'!$B$2:$B$99,A5)</f>
+        <v>35</v>
       </c>
       <c r="C5" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A5,'Daftar Fitur'!$E$2:$E$100,"Ada")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A5,'Daftar Fitur'!$E$2:$E$99,"Ada")</f>
         <v>22</v>
       </c>
       <c r="D5" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A5,'Daftar Fitur'!$E$2:$E$100,"Belum")</f>
-        <v>14</v>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A5,'Daftar Fitur'!$E$2:$E$99,"Belum")</f>
+        <v>13</v>
       </c>
       <c r="E5" s="6" t="n">
         <f aca="false">IF(B5=0,0,C5/B5)</f>
-        <v>0.611111111111111</v>
+        <v>0.628571428571429</v>
       </c>
       <c r="F5" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A5,'Daftar Fitur'!$F$2:$F$100,"Ya")</f>
-        <v>5</v>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A5,'Daftar Fitur'!$F$2:$F$99,"Ya")</f>
+        <v>4</v>
       </c>
       <c r="G5" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A5,'Daftar Fitur'!$F$2:$F$100,"Ya",'Daftar Fitur'!$E$2:$E$100,"Belum")</f>
-        <v>4</v>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A5,'Daftar Fitur'!$F$2:$F$99,"Ya",'Daftar Fitur'!$E$2:$E$99,"Belum")</f>
+        <v>3</v>
       </c>
       <c r="H5" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A5,'Daftar Fitur'!$G$2:$G$100,"Ya")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A5,'Daftar Fitur'!$G$2:$G$99,"Ya")</f>
         <v>8</v>
       </c>
     </row>
@@ -1933,15 +1924,15 @@
         <v>11</v>
       </c>
       <c r="B6" s="5" t="n">
-        <f aca="false">COUNTIF('Daftar Fitur'!$B$2:$B$100,A6)</f>
+        <f aca="false">COUNTIF('Daftar Fitur'!$B$2:$B$99,A6)</f>
         <v>41</v>
       </c>
       <c r="C6" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A6,'Daftar Fitur'!$E$2:$E$100,"Ada")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A6,'Daftar Fitur'!$E$2:$E$99,"Ada")</f>
         <v>21</v>
       </c>
       <c r="D6" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A6,'Daftar Fitur'!$E$2:$E$100,"Belum")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A6,'Daftar Fitur'!$E$2:$E$99,"Belum")</f>
         <v>20</v>
       </c>
       <c r="E6" s="6" t="n">
@@ -1949,15 +1940,15 @@
         <v>0.51219512195122</v>
       </c>
       <c r="F6" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A6,'Daftar Fitur'!$F$2:$F$100,"Ya")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A6,'Daftar Fitur'!$F$2:$F$99,"Ya")</f>
         <v>10</v>
       </c>
       <c r="G6" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A6,'Daftar Fitur'!$F$2:$F$100,"Ya",'Daftar Fitur'!$E$2:$E$100,"Belum")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A6,'Daftar Fitur'!$F$2:$F$99,"Ya",'Daftar Fitur'!$E$2:$E$99,"Belum")</f>
         <v>8</v>
       </c>
       <c r="H6" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A6,'Daftar Fitur'!$G$2:$G$100,"Ya")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A6,'Daftar Fitur'!$G$2:$G$99,"Ya")</f>
         <v>8</v>
       </c>
     </row>
@@ -1966,15 +1957,15 @@
         <v>12</v>
       </c>
       <c r="B7" s="5" t="n">
-        <f aca="false">COUNTIF('Daftar Fitur'!$B$2:$B$100,A7)</f>
+        <f aca="false">COUNTIF('Daftar Fitur'!$B$2:$B$99,A7)</f>
         <v>22</v>
       </c>
       <c r="C7" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A7,'Daftar Fitur'!$E$2:$E$100,"Ada")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A7,'Daftar Fitur'!$E$2:$E$99,"Ada")</f>
         <v>9</v>
       </c>
       <c r="D7" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A7,'Daftar Fitur'!$E$2:$E$100,"Belum")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A7,'Daftar Fitur'!$E$2:$E$99,"Belum")</f>
         <v>13</v>
       </c>
       <c r="E7" s="6" t="n">
@@ -1982,15 +1973,15 @@
         <v>0.409090909090909</v>
       </c>
       <c r="F7" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A7,'Daftar Fitur'!$F$2:$F$100,"Ya")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A7,'Daftar Fitur'!$F$2:$F$99,"Ya")</f>
         <v>2</v>
       </c>
       <c r="G7" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A7,'Daftar Fitur'!$F$2:$F$100,"Ya",'Daftar Fitur'!$E$2:$E$100,"Belum")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A7,'Daftar Fitur'!$F$2:$F$99,"Ya",'Daftar Fitur'!$E$2:$E$99,"Belum")</f>
         <v>2</v>
       </c>
       <c r="H7" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$100,A7,'Daftar Fitur'!$G$2:$G$100,"Ya")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A7,'Daftar Fitur'!$G$2:$G$99,"Ya")</f>
         <v>0</v>
       </c>
     </row>
@@ -2000,7 +1991,7 @@
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">SUM(B5:B7)</f>
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C8" s="8" t="n">
         <f aca="false">SUM(C5:C7)</f>
@@ -2008,19 +1999,19 @@
       </c>
       <c r="D8" s="8" t="n">
         <f aca="false">SUM(D5:D7)</f>
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E8" s="9" t="n">
         <f aca="false">IF(B8=0,0,C8/B8)</f>
-        <v>0.525252525252525</v>
+        <v>0.530612244897959</v>
       </c>
       <c r="F8" s="8" t="n">
         <f aca="false">SUM(F5:F7)</f>
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G8" s="8" t="n">
         <f aca="false">SUM(G5:G7)</f>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H8" s="8" t="n">
         <f aca="false">SUM(H5:H7)</f>
@@ -2096,7 +2087,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K100"/>
+  <dimension ref="A1:K99"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -2845,7 +2836,7 @@
       </c>
       <c r="K25" s="16"/>
     </row>
-    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="n">
         <v>25</v>
       </c>
@@ -2853,25 +2844,25 @@
         <v>10</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>101</v>
+        <v>128</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F26" s="13" t="s">
-        <v>41</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="F26" s="13"/>
       <c r="G26" s="13"/>
       <c r="H26" s="14" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I26" s="14" t="s">
-        <v>130</v>
-      </c>
-      <c r="J26" s="14"/>
+        <v>131</v>
+      </c>
+      <c r="J26" s="14" t="s">
+        <v>132</v>
+      </c>
       <c r="K26" s="16"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2882,10 +2873,10 @@
         <v>10</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E27" s="13" t="s">
         <v>15</v>
@@ -2893,13 +2884,13 @@
       <c r="F27" s="13"/>
       <c r="G27" s="13"/>
       <c r="H27" s="14" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I27" s="14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J27" s="14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="K27" s="16"/>
     </row>
@@ -2911,10 +2902,10 @@
         <v>10</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E28" s="13" t="s">
         <v>15</v>
@@ -2922,13 +2913,13 @@
       <c r="F28" s="13"/>
       <c r="G28" s="13"/>
       <c r="H28" s="14" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I28" s="14" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J28" s="14" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="K28" s="16"/>
     </row>
@@ -2940,10 +2931,10 @@
         <v>10</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E29" s="13" t="s">
         <v>15</v>
@@ -2951,13 +2942,13 @@
       <c r="F29" s="13"/>
       <c r="G29" s="13"/>
       <c r="H29" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I29" s="14" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="J29" s="14" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="K29" s="16"/>
     </row>
@@ -2969,10 +2960,10 @@
         <v>10</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E30" s="13" t="s">
         <v>15</v>
@@ -2980,17 +2971,17 @@
       <c r="F30" s="13"/>
       <c r="G30" s="13"/>
       <c r="H30" s="14" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I30" s="14" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J30" s="14" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="K30" s="16"/>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="n">
         <v>30</v>
       </c>
@@ -2998,10 +2989,10 @@
         <v>10</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E31" s="13" t="s">
         <v>15</v>
@@ -3009,17 +3000,17 @@
       <c r="F31" s="13"/>
       <c r="G31" s="13"/>
       <c r="H31" s="14" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I31" s="14" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J31" s="14" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K31" s="16"/>
     </row>
-    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="n">
         <v>31</v>
       </c>
@@ -3027,10 +3018,10 @@
         <v>10</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E32" s="13" t="s">
         <v>15</v>
@@ -3038,13 +3029,13 @@
       <c r="F32" s="13"/>
       <c r="G32" s="13"/>
       <c r="H32" s="14" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I32" s="14" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J32" s="14" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="K32" s="16"/>
     </row>
@@ -3056,28 +3047,28 @@
         <v>10</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F33" s="13"/>
-      <c r="G33" s="13"/>
+      <c r="G33" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="H33" s="14" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="I33" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="J33" s="14" t="s">
         <v>159</v>
       </c>
+      <c r="J33" s="14"/>
       <c r="K33" s="16"/>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="n">
         <v>33</v>
       </c>
@@ -3085,25 +3076,27 @@
         <v>10</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>131</v>
+        <v>160</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F34" s="13"/>
       <c r="G34" s="13" t="s">
         <v>41</v>
       </c>
       <c r="H34" s="14" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="I34" s="14" t="s">
-        <v>162</v>
-      </c>
-      <c r="J34" s="14"/>
+        <v>163</v>
+      </c>
+      <c r="J34" s="14" t="s">
+        <v>164</v>
+      </c>
       <c r="K34" s="16"/>
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3114,27 +3107,25 @@
         <v>10</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F35" s="13"/>
       <c r="G35" s="13" t="s">
         <v>41</v>
       </c>
       <c r="H35" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I35" s="14" t="s">
-        <v>166</v>
-      </c>
-      <c r="J35" s="14" t="s">
         <v>167</v>
       </c>
+      <c r="J35" s="14"/>
       <c r="K35" s="16"/>
     </row>
     <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3145,7 +3136,7 @@
         <v>10</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D36" s="15" t="s">
         <v>168</v>
@@ -3171,28 +3162,30 @@
         <v>36</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F37" s="13"/>
       <c r="G37" s="13" t="s">
         <v>41</v>
       </c>
       <c r="H37" s="14" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="I37" s="14" t="s">
-        <v>173</v>
-      </c>
-      <c r="J37" s="14"/>
+        <v>174</v>
+      </c>
+      <c r="J37" s="14" t="s">
+        <v>175</v>
+      </c>
       <c r="K37" s="16"/>
     </row>
     <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3203,26 +3196,24 @@
         <v>11</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D38" s="15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>15</v>
       </c>
       <c r="F38" s="13"/>
-      <c r="G38" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="G38" s="13"/>
       <c r="H38" s="14" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I38" s="14" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J38" s="14" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K38" s="16"/>
     </row>
@@ -3234,10 +3225,10 @@
         <v>11</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D39" s="15" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E39" s="13" t="s">
         <v>15</v>
@@ -3245,13 +3236,13 @@
       <c r="F39" s="13"/>
       <c r="G39" s="13"/>
       <c r="H39" s="14" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="I39" s="14" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J39" s="14" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K39" s="16"/>
     </row>
@@ -3263,25 +3254,25 @@
         <v>11</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D40" s="15" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F40" s="13"/>
-      <c r="G40" s="13"/>
+      <c r="G40" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="H40" s="14" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I40" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="J40" s="14" t="s">
         <v>186</v>
       </c>
+      <c r="J40" s="14"/>
       <c r="K40" s="16"/>
     </row>
     <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3292,7 +3283,7 @@
         <v>11</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D41" s="15" t="s">
         <v>187</v>
@@ -3300,10 +3291,10 @@
       <c r="E41" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F41" s="13"/>
-      <c r="G41" s="13" t="s">
+      <c r="F41" s="13" t="s">
         <v>41</v>
       </c>
+      <c r="G41" s="13"/>
       <c r="H41" s="14" t="s">
         <v>188</v>
       </c>
@@ -3321,7 +3312,7 @@
         <v>11</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D42" s="15" t="s">
         <v>190</v>
@@ -3329,9 +3320,7 @@
       <c r="E42" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F42" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="F42" s="13"/>
       <c r="G42" s="13"/>
       <c r="H42" s="14" t="s">
         <v>191</v>
@@ -3339,7 +3328,9 @@
       <c r="I42" s="14" t="s">
         <v>192</v>
       </c>
-      <c r="J42" s="14"/>
+      <c r="J42" s="14" t="s">
+        <v>193</v>
+      </c>
       <c r="K42" s="16"/>
     </row>
     <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3350,24 +3341,24 @@
         <v>11</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>174</v>
+        <v>194</v>
       </c>
       <c r="D43" s="15" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="E43" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F43" s="13"/>
       <c r="G43" s="13"/>
       <c r="H43" s="14" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="I43" s="14" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="J43" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="K43" s="16"/>
     </row>
@@ -3379,10 +3370,10 @@
         <v>11</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D44" s="15" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E44" s="13" t="s">
         <v>15</v>
@@ -3390,13 +3381,13 @@
       <c r="F44" s="13"/>
       <c r="G44" s="13"/>
       <c r="H44" s="14" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="I44" s="14" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="J44" s="14" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="K44" s="16"/>
     </row>
@@ -3408,10 +3399,10 @@
         <v>11</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D45" s="15" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E45" s="13" t="s">
         <v>15</v>
@@ -3419,13 +3410,13 @@
       <c r="F45" s="13"/>
       <c r="G45" s="13"/>
       <c r="H45" s="14" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I45" s="14" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="J45" s="14" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="K45" s="16"/>
     </row>
@@ -3437,10 +3428,10 @@
         <v>11</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D46" s="15" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E46" s="13" t="s">
         <v>15</v>
@@ -3448,13 +3439,13 @@
       <c r="F46" s="13"/>
       <c r="G46" s="13"/>
       <c r="H46" s="14" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I46" s="14" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="J46" s="14" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K46" s="16"/>
     </row>
@@ -3466,24 +3457,28 @@
         <v>11</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D47" s="15" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E47" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="F47" s="13"/>
-      <c r="G47" s="13"/>
+      <c r="F47" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="G47" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="H47" s="14" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="I47" s="14" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J47" s="14" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="K47" s="16"/>
     </row>
@@ -3495,28 +3490,24 @@
         <v>11</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D48" s="15" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E48" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="F48" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="G48" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="F48" s="13"/>
+      <c r="G48" s="13"/>
       <c r="H48" s="14" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="I48" s="14" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J48" s="14" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="K48" s="16"/>
     </row>
@@ -3528,25 +3519,25 @@
         <v>11</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D49" s="15" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E49" s="13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F49" s="13"/>
-      <c r="G49" s="13"/>
+      <c r="G49" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="H49" s="14" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="I49" s="14" t="s">
-        <v>220</v>
-      </c>
-      <c r="J49" s="14" t="s">
         <v>221</v>
       </c>
+      <c r="J49" s="14"/>
       <c r="K49" s="16"/>
     </row>
     <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3557,7 +3548,7 @@
         <v>11</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D50" s="15" t="s">
         <v>222</v>
@@ -3566,9 +3557,7 @@
         <v>17</v>
       </c>
       <c r="F50" s="13"/>
-      <c r="G50" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="G50" s="13"/>
       <c r="H50" s="14" t="s">
         <v>223</v>
       </c>
@@ -3586,7 +3575,7 @@
         <v>11</v>
       </c>
       <c r="C51" s="14" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D51" s="15" t="s">
         <v>225</v>
@@ -3613,7 +3602,7 @@
         <v>11</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D52" s="15" t="s">
         <v>228</v>
@@ -3621,7 +3610,9 @@
       <c r="E52" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F52" s="13"/>
+      <c r="F52" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="G52" s="13"/>
       <c r="H52" s="14" t="s">
         <v>229</v>
@@ -3640,7 +3631,7 @@
         <v>11</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D53" s="15" t="s">
         <v>231</v>
@@ -3669,25 +3660,27 @@
         <v>11</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>197</v>
+        <v>234</v>
       </c>
       <c r="D54" s="15" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E54" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F54" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F54" s="13"/>
+      <c r="G54" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="G54" s="13"/>
       <c r="H54" s="14" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="I54" s="14" t="s">
-        <v>236</v>
-      </c>
-      <c r="J54" s="14"/>
+        <v>237</v>
+      </c>
+      <c r="J54" s="14" t="s">
+        <v>238</v>
+      </c>
       <c r="K54" s="16"/>
     </row>
     <row r="55" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3698,26 +3691,24 @@
         <v>11</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D55" s="15" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E55" s="13" t="s">
         <v>15</v>
       </c>
       <c r="F55" s="13"/>
-      <c r="G55" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="G55" s="13"/>
       <c r="H55" s="14" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="I55" s="14" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J55" s="14" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="K55" s="16"/>
     </row>
@@ -3729,24 +3720,26 @@
         <v>11</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D56" s="15" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E56" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="F56" s="13"/>
+      <c r="F56" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="G56" s="13"/>
       <c r="H56" s="14" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="I56" s="14" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="J56" s="14" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="K56" s="16"/>
     </row>
@@ -3758,26 +3751,24 @@
         <v>11</v>
       </c>
       <c r="C57" s="14" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D57" s="15" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E57" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="F57" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="F57" s="13"/>
       <c r="G57" s="13"/>
       <c r="H57" s="14" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="I57" s="14" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="J57" s="14" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="K57" s="16"/>
     </row>
@@ -3789,10 +3780,10 @@
         <v>11</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D58" s="15" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E58" s="13" t="s">
         <v>15</v>
@@ -3800,13 +3791,13 @@
       <c r="F58" s="13"/>
       <c r="G58" s="13"/>
       <c r="H58" s="14" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="I58" s="14" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="J58" s="14" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="K58" s="16"/>
     </row>
@@ -3818,10 +3809,10 @@
         <v>11</v>
       </c>
       <c r="C59" s="14" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D59" s="15" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E59" s="13" t="s">
         <v>15</v>
@@ -3829,13 +3820,13 @@
       <c r="F59" s="13"/>
       <c r="G59" s="13"/>
       <c r="H59" s="14" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="I59" s="14" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="J59" s="14" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="K59" s="16"/>
     </row>
@@ -3847,10 +3838,10 @@
         <v>11</v>
       </c>
       <c r="C60" s="14" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D60" s="15" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E60" s="13" t="s">
         <v>15</v>
@@ -3858,13 +3849,13 @@
       <c r="F60" s="13"/>
       <c r="G60" s="13"/>
       <c r="H60" s="14" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="I60" s="14" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="J60" s="14" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="K60" s="16"/>
     </row>
@@ -3876,10 +3867,10 @@
         <v>11</v>
       </c>
       <c r="C61" s="14" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D61" s="15" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E61" s="13" t="s">
         <v>15</v>
@@ -3887,13 +3878,13 @@
       <c r="F61" s="13"/>
       <c r="G61" s="13"/>
       <c r="H61" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="I61" s="14" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="J61" s="14" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="K61" s="16"/>
     </row>
@@ -3905,25 +3896,23 @@
         <v>11</v>
       </c>
       <c r="C62" s="14" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D62" s="15" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E62" s="13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F62" s="13"/>
       <c r="G62" s="13"/>
       <c r="H62" s="14" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I62" s="14" t="s">
-        <v>268</v>
-      </c>
-      <c r="J62" s="14" t="s">
         <v>269</v>
       </c>
+      <c r="J62" s="14"/>
       <c r="K62" s="16"/>
     </row>
     <row r="63" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3934,7 +3923,7 @@
         <v>11</v>
       </c>
       <c r="C63" s="14" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D63" s="15" t="s">
         <v>270</v>
@@ -3943,7 +3932,9 @@
         <v>17</v>
       </c>
       <c r="F63" s="13"/>
-      <c r="G63" s="13"/>
+      <c r="G63" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="H63" s="14" t="s">
         <v>271</v>
       </c>
@@ -3961,7 +3952,7 @@
         <v>11</v>
       </c>
       <c r="C64" s="14" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D64" s="15" t="s">
         <v>273</v>
@@ -3970,9 +3961,7 @@
         <v>17</v>
       </c>
       <c r="F64" s="13"/>
-      <c r="G64" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="G64" s="13"/>
       <c r="H64" s="14" t="s">
         <v>274</v>
       </c>
@@ -3990,23 +3979,25 @@
         <v>11</v>
       </c>
       <c r="C65" s="14" t="s">
-        <v>237</v>
+        <v>276</v>
       </c>
       <c r="D65" s="15" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E65" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F65" s="13"/>
       <c r="G65" s="13"/>
       <c r="H65" s="14" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="I65" s="14" t="s">
-        <v>278</v>
-      </c>
-      <c r="J65" s="14"/>
+        <v>279</v>
+      </c>
+      <c r="J65" s="14" t="s">
+        <v>280</v>
+      </c>
       <c r="K65" s="16"/>
     </row>
     <row r="66" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4017,10 +4008,10 @@
         <v>11</v>
       </c>
       <c r="C66" s="14" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="D66" s="15" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E66" s="13" t="s">
         <v>15</v>
@@ -4028,13 +4019,13 @@
       <c r="F66" s="13"/>
       <c r="G66" s="13"/>
       <c r="H66" s="14" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="I66" s="14" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="J66" s="14" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="K66" s="16"/>
     </row>
@@ -4046,10 +4037,10 @@
         <v>11</v>
       </c>
       <c r="C67" s="14" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="D67" s="15" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E67" s="13" t="s">
         <v>15</v>
@@ -4057,13 +4048,13 @@
       <c r="F67" s="13"/>
       <c r="G67" s="13"/>
       <c r="H67" s="14" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="I67" s="14" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="J67" s="14" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="K67" s="16"/>
     </row>
@@ -4075,25 +4066,25 @@
         <v>11</v>
       </c>
       <c r="C68" s="14" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="D68" s="15" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E68" s="13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F68" s="13"/>
-      <c r="G68" s="13"/>
+      <c r="G68" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="H68" s="14" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="I68" s="14" t="s">
-        <v>290</v>
-      </c>
-      <c r="J68" s="14" t="s">
         <v>291</v>
       </c>
+      <c r="J68" s="14"/>
       <c r="K68" s="16"/>
     </row>
     <row r="69" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4104,28 +4095,28 @@
         <v>11</v>
       </c>
       <c r="C69" s="14" t="s">
-        <v>279</v>
+        <v>292</v>
       </c>
       <c r="D69" s="15" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E69" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F69" s="13"/>
-      <c r="G69" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="G69" s="13"/>
       <c r="H69" s="14" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="I69" s="14" t="s">
-        <v>294</v>
-      </c>
-      <c r="J69" s="14"/>
+        <v>295</v>
+      </c>
+      <c r="J69" s="14" t="s">
+        <v>296</v>
+      </c>
       <c r="K69" s="16"/>
     </row>
-    <row r="70" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="13" t="n">
         <v>69</v>
       </c>
@@ -4133,28 +4124,30 @@
         <v>11</v>
       </c>
       <c r="C70" s="14" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="D70" s="15" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E70" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F70" s="13"/>
-      <c r="G70" s="13"/>
+        <v>17</v>
+      </c>
+      <c r="F70" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="G70" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="H70" s="14" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="I70" s="14" t="s">
-        <v>298</v>
-      </c>
-      <c r="J70" s="14" t="s">
         <v>299</v>
       </c>
+      <c r="J70" s="14"/>
       <c r="K70" s="16"/>
     </row>
-    <row r="71" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="13" t="n">
         <v>70</v>
       </c>
@@ -4162,7 +4155,7 @@
         <v>11</v>
       </c>
       <c r="C71" s="14" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="D71" s="15" t="s">
         <v>300</v>
@@ -4173,9 +4166,7 @@
       <c r="F71" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="G71" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="G71" s="13"/>
       <c r="H71" s="14" t="s">
         <v>301</v>
       </c>
@@ -4193,7 +4184,7 @@
         <v>11</v>
       </c>
       <c r="C72" s="14" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="D72" s="15" t="s">
         <v>303</v>
@@ -4201,9 +4192,7 @@
       <c r="E72" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F72" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="F72" s="13"/>
       <c r="G72" s="13"/>
       <c r="H72" s="14" t="s">
         <v>304</v>
@@ -4222,7 +4211,7 @@
         <v>11</v>
       </c>
       <c r="C73" s="14" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="D73" s="15" t="s">
         <v>306</v>
@@ -4230,7 +4219,9 @@
       <c r="E73" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F73" s="13"/>
+      <c r="F73" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="G73" s="13"/>
       <c r="H73" s="14" t="s">
         <v>307</v>
@@ -4249,7 +4240,7 @@
         <v>11</v>
       </c>
       <c r="C74" s="14" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="D74" s="15" t="s">
         <v>309</v>
@@ -4257,9 +4248,7 @@
       <c r="E74" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F74" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="F74" s="13"/>
       <c r="G74" s="13"/>
       <c r="H74" s="14" t="s">
         <v>310</v>
@@ -4278,7 +4267,7 @@
         <v>11</v>
       </c>
       <c r="C75" s="14" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="D75" s="15" t="s">
         <v>312</v>
@@ -4286,7 +4275,9 @@
       <c r="E75" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F75" s="13"/>
+      <c r="F75" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="G75" s="13"/>
       <c r="H75" s="14" t="s">
         <v>313</v>
@@ -4297,7 +4288,7 @@
       <c r="J75" s="14"/>
       <c r="K75" s="16"/>
     </row>
-    <row r="76" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="13" t="n">
         <v>75</v>
       </c>
@@ -4305,7 +4296,7 @@
         <v>11</v>
       </c>
       <c r="C76" s="14" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="D76" s="15" t="s">
         <v>315</v>
@@ -4326,7 +4317,7 @@
       <c r="J76" s="14"/>
       <c r="K76" s="16"/>
     </row>
-    <row r="77" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="13" t="n">
         <v>76</v>
       </c>
@@ -4334,7 +4325,7 @@
         <v>11</v>
       </c>
       <c r="C77" s="14" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="D77" s="15" t="s">
         <v>318</v>
@@ -4342,9 +4333,7 @@
       <c r="E77" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F77" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="F77" s="13"/>
       <c r="G77" s="13"/>
       <c r="H77" s="14" t="s">
         <v>319</v>
@@ -4360,26 +4349,28 @@
         <v>77</v>
       </c>
       <c r="B78" s="14" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C78" s="14" t="s">
-        <v>295</v>
+        <v>321</v>
       </c>
       <c r="D78" s="15" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E78" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F78" s="13"/>
       <c r="G78" s="13"/>
       <c r="H78" s="14" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="I78" s="14" t="s">
-        <v>323</v>
-      </c>
-      <c r="J78" s="14"/>
+        <v>324</v>
+      </c>
+      <c r="J78" s="14" t="s">
+        <v>325</v>
+      </c>
       <c r="K78" s="16"/>
     </row>
     <row r="79" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4390,25 +4381,23 @@
         <v>12</v>
       </c>
       <c r="C79" s="14" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="D79" s="15" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E79" s="13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F79" s="13"/>
       <c r="G79" s="13"/>
       <c r="H79" s="14" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="I79" s="14" t="s">
-        <v>327</v>
-      </c>
-      <c r="J79" s="14" t="s">
         <v>328</v>
       </c>
+      <c r="J79" s="14"/>
       <c r="K79" s="16"/>
     </row>
     <row r="80" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4419,7 +4408,7 @@
         <v>12</v>
       </c>
       <c r="C80" s="14" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="D80" s="15" t="s">
         <v>329</v>
@@ -4427,7 +4416,9 @@
       <c r="E80" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F80" s="13"/>
+      <c r="F80" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="G80" s="13"/>
       <c r="H80" s="14" t="s">
         <v>330</v>
@@ -4446,25 +4437,25 @@
         <v>12</v>
       </c>
       <c r="C81" s="14" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
       <c r="D81" s="15" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E81" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F81" s="13" t="s">
-        <v>41</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="F81" s="13"/>
       <c r="G81" s="13"/>
       <c r="H81" s="14" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="I81" s="14" t="s">
-        <v>334</v>
-      </c>
-      <c r="J81" s="14"/>
+        <v>335</v>
+      </c>
+      <c r="J81" s="14" t="s">
+        <v>336</v>
+      </c>
       <c r="K81" s="16"/>
     </row>
     <row r="82" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4475,10 +4466,10 @@
         <v>12</v>
       </c>
       <c r="C82" s="14" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="D82" s="15" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E82" s="13" t="s">
         <v>15</v>
@@ -4486,13 +4477,13 @@
       <c r="F82" s="13"/>
       <c r="G82" s="13"/>
       <c r="H82" s="14" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="I82" s="14" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="J82" s="14" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="K82" s="16"/>
     </row>
@@ -4504,25 +4495,23 @@
         <v>12</v>
       </c>
       <c r="C83" s="14" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="D83" s="15" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="E83" s="13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F83" s="13"/>
       <c r="G83" s="13"/>
       <c r="H83" s="14" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="I83" s="14" t="s">
-        <v>342</v>
-      </c>
-      <c r="J83" s="14" t="s">
         <v>343</v>
       </c>
+      <c r="J83" s="14"/>
       <c r="K83" s="16"/>
     </row>
     <row r="84" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4533,7 +4522,7 @@
         <v>12</v>
       </c>
       <c r="C84" s="14" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="D84" s="15" t="s">
         <v>344</v>
@@ -4541,7 +4530,9 @@
       <c r="E84" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F84" s="13"/>
+      <c r="F84" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="G84" s="13"/>
       <c r="H84" s="14" t="s">
         <v>345</v>
@@ -4560,25 +4551,25 @@
         <v>12</v>
       </c>
       <c r="C85" s="14" t="s">
-        <v>335</v>
+        <v>347</v>
       </c>
       <c r="D85" s="15" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E85" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F85" s="13" t="s">
-        <v>41</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="F85" s="13"/>
       <c r="G85" s="13"/>
       <c r="H85" s="14" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="I85" s="14" t="s">
-        <v>349</v>
-      </c>
-      <c r="J85" s="14"/>
+        <v>350</v>
+      </c>
+      <c r="J85" s="14" t="s">
+        <v>351</v>
+      </c>
       <c r="K85" s="16"/>
     </row>
     <row r="86" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4589,25 +4580,23 @@
         <v>12</v>
       </c>
       <c r="C86" s="14" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="D86" s="15" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E86" s="13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F86" s="13"/>
       <c r="G86" s="13"/>
       <c r="H86" s="14" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="I86" s="14" t="s">
-        <v>353</v>
-      </c>
-      <c r="J86" s="14" t="s">
         <v>354</v>
       </c>
+      <c r="J86" s="14"/>
       <c r="K86" s="16"/>
     </row>
     <row r="87" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4618,7 +4607,7 @@
         <v>12</v>
       </c>
       <c r="C87" s="14" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="D87" s="15" t="s">
         <v>355</v>
@@ -4645,7 +4634,7 @@
         <v>12</v>
       </c>
       <c r="C88" s="14" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="D88" s="15" t="s">
         <v>358</v>
@@ -4672,7 +4661,7 @@
         <v>12</v>
       </c>
       <c r="C89" s="14" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="D89" s="15" t="s">
         <v>361</v>
@@ -4699,23 +4688,25 @@
         <v>12</v>
       </c>
       <c r="C90" s="14" t="s">
-        <v>350</v>
+        <v>364</v>
       </c>
       <c r="D90" s="15" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E90" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F90" s="13"/>
       <c r="G90" s="13"/>
       <c r="H90" s="14" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="I90" s="14" t="s">
-        <v>366</v>
-      </c>
-      <c r="J90" s="14"/>
+        <v>367</v>
+      </c>
+      <c r="J90" s="14" t="s">
+        <v>368</v>
+      </c>
       <c r="K90" s="16"/>
     </row>
     <row r="91" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4726,10 +4717,10 @@
         <v>12</v>
       </c>
       <c r="C91" s="14" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="D91" s="15" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E91" s="13" t="s">
         <v>15</v>
@@ -4737,13 +4728,13 @@
       <c r="F91" s="13"/>
       <c r="G91" s="13"/>
       <c r="H91" s="14" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="I91" s="14" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="J91" s="14" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="K91" s="16"/>
     </row>
@@ -4755,10 +4746,10 @@
         <v>12</v>
       </c>
       <c r="C92" s="14" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="D92" s="15" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E92" s="13" t="s">
         <v>15</v>
@@ -4766,13 +4757,13 @@
       <c r="F92" s="13"/>
       <c r="G92" s="13"/>
       <c r="H92" s="14" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="I92" s="14" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="J92" s="14" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="K92" s="16"/>
     </row>
@@ -4784,10 +4775,10 @@
         <v>12</v>
       </c>
       <c r="C93" s="14" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="D93" s="15" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E93" s="13" t="s">
         <v>15</v>
@@ -4795,13 +4786,13 @@
       <c r="F93" s="13"/>
       <c r="G93" s="13"/>
       <c r="H93" s="14" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="I93" s="14" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="J93" s="14" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="K93" s="16"/>
     </row>
@@ -4813,25 +4804,23 @@
         <v>12</v>
       </c>
       <c r="C94" s="14" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="D94" s="15" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="E94" s="13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F94" s="13"/>
       <c r="G94" s="13"/>
       <c r="H94" s="14" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="I94" s="14" t="s">
-        <v>382</v>
-      </c>
-      <c r="J94" s="14" t="s">
         <v>383</v>
       </c>
+      <c r="J94" s="14"/>
       <c r="K94" s="16"/>
     </row>
     <row r="95" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4842,7 +4831,7 @@
         <v>12</v>
       </c>
       <c r="C95" s="14" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="D95" s="15" t="s">
         <v>384</v>
@@ -4869,7 +4858,7 @@
         <v>12</v>
       </c>
       <c r="C96" s="14" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="D96" s="15" t="s">
         <v>387</v>
@@ -4896,10 +4885,10 @@
         <v>12</v>
       </c>
       <c r="C97" s="14" t="s">
-        <v>367</v>
+        <v>390</v>
       </c>
       <c r="D97" s="15" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="E97" s="13" t="s">
         <v>17</v>
@@ -4907,10 +4896,10 @@
       <c r="F97" s="13"/>
       <c r="G97" s="13"/>
       <c r="H97" s="14" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="I97" s="14" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="J97" s="14"/>
       <c r="K97" s="16"/>
@@ -4923,7 +4912,7 @@
         <v>12</v>
       </c>
       <c r="C98" s="14" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="D98" s="15" t="s">
         <v>394</v>
@@ -4939,7 +4928,9 @@
       <c r="I98" s="14" t="s">
         <v>396</v>
       </c>
-      <c r="J98" s="14"/>
+      <c r="J98" s="14" t="s">
+        <v>397</v>
+      </c>
       <c r="K98" s="16"/>
     </row>
     <row r="99" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4950,59 +4941,30 @@
         <v>12</v>
       </c>
       <c r="C99" s="14" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="D99" s="15" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E99" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F99" s="13"/>
       <c r="G99" s="13"/>
       <c r="H99" s="14" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="I99" s="14" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="J99" s="14" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K99" s="16"/>
     </row>
-    <row r="100" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="13" t="n">
-        <v>99</v>
-      </c>
-      <c r="B100" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="C100" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="D100" s="15" t="s">
-        <v>401</v>
-      </c>
-      <c r="E100" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F100" s="13"/>
-      <c r="G100" s="13"/>
-      <c r="H100" s="14" t="s">
-        <v>402</v>
-      </c>
-      <c r="I100" s="14" t="s">
-        <v>403</v>
-      </c>
-      <c r="J100" s="14" t="s">
-        <v>404</v>
-      </c>
-      <c r="K100" s="16"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K100"/>
-  <conditionalFormatting sqref="E2:E100">
+  <autoFilter ref="A1:K99"/>
+  <conditionalFormatting sqref="E2:E99">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"Ada"</formula>
     </cfRule>
@@ -5011,11 +4973,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E100" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E99" type="list">
       <formula1>"Ada,Belum,Sebagian"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K2:K100" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K2:K99" type="list">
       <formula1>"P1 - Quick win,P2 - Pembeda,P3 - Naik kelas,P4 - Skala"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -5045,42 +5007,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dokumen rancangan: 96 fitur (foto->produk AI dan kasir POS dikeluarkan), semua bertanda sudah dibangun beserta lokasinya di kode, catatan pemasangan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HmiNd1QbTyjAfj7oGbYGxq
</commit_message>
<xml_diff>
--- a/docs/rancangan-fitur-marketplace-umkm.xlsx
+++ b/docs/rancangan-fitur-marketplace-umkm.xlsx
@@ -10,10 +10,10 @@
   <sheets>
     <sheet name="Ringkasan" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Daftar Fitur" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Roadmap" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Catatan Pemasangan" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Daftar Fitur'!$A$1:$K$99</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Daftar Fitur'!$A$1:$K$97</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="750" uniqueCount="445">
   <si>
     <t xml:space="preserve">Rancangan Fitur Marketplace UMKM — Gap Analysis Repository myumkm</t>
   </si>
@@ -99,7 +99,7 @@
     <t xml:space="preserve">Sumber</t>
   </si>
   <si>
-    <t xml:space="preserve">Analisis kode repo xaralien/myumkm (CodeIgniter 3), per 13 Okt 2026. Dibaca dari kode, aplikasi tidak dijalankan.</t>
+    <t xml:space="preserve">Analisis kode repo xaralien/myumkm (CodeIgniter 3), per 13 Okt 2026, setelah semua fitur dibangun &amp; diuji di lingkungan lokal.</t>
   </si>
   <si>
     <t xml:space="preserve">No</t>
@@ -183,6 +183,9 @@
     <t xml:space="preserve">Masuk cukup dengan kode OTP dikirim ke WA.</t>
   </si>
   <si>
+    <t xml:space="preserve">Auth::otp + Auth_lib::buat_token — kode 6 angka dikirim lewat gerbang WA.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lupa kata sandi mandiri</t>
   </si>
   <si>
@@ -192,7 +195,7 @@
     <t xml:space="preserve">Tautan/OTP reset sandi sendiri.</t>
   </si>
   <si>
-    <t xml:space="preserve">Repo hanya punya reset oleh admin: admin/Users::sandi</t>
+    <t xml:space="preserve">Auth::lupa / Auth::reset — tautan reset via WA/email, token sekali pakai.</t>
   </si>
   <si>
     <t xml:space="preserve">Profil &amp; ubah sandi</t>
@@ -291,6 +294,9 @@
     <t xml:space="preserve">Tombol ♥ dan daftar favorit.</t>
   </si>
   <si>
+    <t xml:space="preserve">Favorit controller, tabel wishlists, tombol ♥ di kartu &amp; halaman produk.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ikuti toko</t>
   </si>
   <si>
@@ -300,6 +306,9 @@
     <t xml:space="preserve">Follow toko + kabar produk baru.</t>
   </si>
   <si>
+    <t xml:space="preserve">Favorit::ikuti, tabel store_follows; deret "Baru dari toko yang kamu ikuti" di beranda.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Rekomendasi &amp; "terlaris"</t>
   </si>
   <si>
@@ -309,6 +318,9 @@
     <t xml:space="preserve">Rekomendasi berdasarkan riwayat, label terlaris di sekitar.</t>
   </si>
   <si>
+    <t xml:space="preserve">urutan terlaris di katalog (kolom terjual_count), deret rekomendasi dari riwayat beli di beranda.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Label "Produk Lokal / Halal / P-IRT / Buatan Tangan"</t>
   </si>
   <si>
@@ -318,6 +330,9 @@
     <t xml:space="preserve">Lencana terverifikasi di kartu produk.</t>
   </si>
   <si>
+    <t xml:space="preserve">kolom buatan_tangan, bahan_lokal, halal_no, pirt_no + lencana; P-IRT/Halal terverifikasi admin.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bagikan produk ke WhatsApp</t>
   </si>
   <si>
@@ -327,7 +342,7 @@
     <t xml:space="preserve">Tombol share dengan pesan siap kirim.</t>
   </si>
   <si>
-    <t xml:space="preserve">Ada kode tombol WA di v_produk.php tapi dikomentari</t>
+    <t xml:space="preserve">parts/bagikan.php — tombol WA dengan pesan siap kirim + salin tautan.</t>
   </si>
   <si>
     <t xml:space="preserve">Keranjang, Checkout &amp; Pembayaran</t>
@@ -390,6 +405,9 @@
     <t xml:space="preserve">Kode voucher toko/platform.</t>
   </si>
   <si>
+    <t xml:space="preserve">Voucher_lib — kode voucher toko &amp; platform di checkout.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Checkout multi-toko</t>
   </si>
   <si>
@@ -399,6 +417,9 @@
     <t xml:space="preserve">Beli dari beberapa toko dalam satu pembayaran.</t>
   </si>
   <si>
+    <t xml:space="preserve">Cart_lib::per_toko + Tagihan_lib — satu pembayaran Duitku (prefiks TG-) untuk banyak toko.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pre-order fleksibel (DP, tanggal ambil, kuota)</t>
   </si>
   <si>
@@ -408,7 +429,7 @@
     <t xml:space="preserve">Pilih tanggal kirim/ambil, bayar DP, kuota harian.</t>
   </si>
   <si>
-    <t xml:space="preserve">Repo baru punya waktu_proses_hari di level toko</t>
+    <t xml:space="preserve">tanggal kirim, kuota harian, DP + pelunasan (Checkout::lunasi).</t>
   </si>
   <si>
     <t xml:space="preserve">Pasca-Pembelian</t>
@@ -507,6 +528,9 @@
     <t xml:space="preserve">Kabar status pesanan dikirim ke WA.</t>
   </si>
   <si>
+    <t xml:space="preserve">Notifikasi_lib — WA (format Fonnte) &amp; email; aktifkan di Admin &gt; Pengaturan.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pengalaman &amp; Aksesibilitas</t>
   </si>
   <si>
@@ -531,6 +555,9 @@
     <t xml:space="preserve">Bisa dipasang di layar utama, gambar ringan, cache offline.</t>
   </si>
   <si>
+    <t xml:space="preserve">manifest.webmanifest, sw.js, halaman offline; mode hemat kuota (tanpa font web).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mode huruf besar &amp; bahasa daerah</t>
   </si>
   <si>
@@ -540,6 +567,9 @@
     <t xml:space="preserve">Pengaturan ukuran huruf, pilihan bahasa.</t>
   </si>
   <si>
+    <t xml:space="preserve">Preferensi controller + t(); huruf besar, bahasa Jawa &amp; Sunda.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Onboarding &amp; Profil Toko</t>
   </si>
   <si>
@@ -588,6 +618,9 @@
     <t xml:space="preserve">Checklist "Toko siap jualan" (foto profil → produk pertama → ongkir → rekening) dengan video 1 menit per langkah.</t>
   </si>
   <si>
+    <t xml:space="preserve">seller/mulai — checklist "Toko siap jualan" + tautan modul Akademi.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bantuan legalitas (NIB, P-IRT, Halal)</t>
   </si>
   <si>
@@ -597,6 +630,9 @@
     <t xml:space="preserve">Panduan langkah-langkah, unggah dokumen, lencana terverifikasi di toko.</t>
   </si>
   <si>
+    <t xml:space="preserve">seller/legalitas — panduan NIB/P-IRT/Halal, unggah dokumen privat, lencana setelah diverifikasi.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mode libur / tutup sementara</t>
   </si>
   <si>
@@ -606,7 +642,7 @@
     <t xml:space="preserve">Toggle libur dengan tanggal buka kembali.</t>
   </si>
   <si>
-    <t xml:space="preserve">Kini hanya admin yang dapat menonaktifkan toko</t>
+    <t xml:space="preserve">seller/libur — tanggal mulai/buka, pesan untuk pembeli, checkout otomatis ditolak.</t>
   </si>
   <si>
     <t xml:space="preserve">Manajemen Produk</t>
@@ -684,15 +720,6 @@
     <t xml:space="preserve">gambar_helper.php, tools/rapikan_gambar_lama.php</t>
   </si>
   <si>
-    <t xml:space="preserve">Tambah produk dari foto saja (AI isi nama, kategori, harga saran)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Form panjang menakutkan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Foto → draf produk lengkap, penjual tinggal konfirmasi.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Peringatan stok menipis</t>
   </si>
   <si>
@@ -702,6 +729,9 @@
     <t xml:space="preserve">Notifikasi saat stok di bawah ambang.</t>
   </si>
   <si>
+    <t xml:space="preserve">ambang di Pengaturan; kabar WA saat pesanan lunas + kartu di dasbor penjual.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Unggah massal (Excel/CSV) &amp; duplikat produk</t>
   </si>
   <si>
@@ -711,6 +741,9 @@
     <t xml:space="preserve">Template Excel sederhana, tombol "duplikat".</t>
   </si>
   <si>
+    <t xml:space="preserve">seller/massal — template .xlsx/.csv, impor &amp; ekspor; tombol duplikat produk.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Harga grosir / minimal beli bertingkat</t>
   </si>
   <si>
@@ -720,6 +753,9 @@
     <t xml:space="preserve">Harga berbeda berdasarkan jumlah.</t>
   </si>
   <si>
+    <t xml:space="preserve">tabel product_tiers, harga otomatis di keranjang.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pengaturan pre-order per produk</t>
   </si>
   <si>
@@ -729,6 +765,9 @@
     <t xml:space="preserve">Lama produksi per produk, kuota harian, DP, kalender tanggal tersedia.</t>
   </si>
   <si>
+    <t xml:space="preserve">kolom is_preorder, po_hari, po_kuota_harian, po_dp_persen.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pesanan &amp; Pengiriman</t>
   </si>
   <si>
@@ -837,6 +876,9 @@
     <t xml:space="preserve">Tarif real-time dan pelacakan otomatis via agregator.</t>
   </si>
   <si>
+    <t xml:space="preserve">Ekspedisi_lib — daftar kurir, lacak resi di halaman pesanan, seller/ongkir bandingkan tarif; perlu kunci agregator (Biteship) di Pengaturan, tanpa kunci tetap ada tautan lacak resmi. Tarif otomatis di checkout pembeli belum.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cetak label pengiriman &amp; nota/struk</t>
   </si>
   <si>
@@ -846,6 +888,9 @@
     <t xml:space="preserve">Cetak label + invoice PDF / printer thermal.</t>
   </si>
   <si>
+    <t xml:space="preserve">seller/cetak — label &amp; nota siap cetak (A4/thermal 58mm).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Notifikasi pesanan baru ke WhatsApp penjual</t>
   </si>
   <si>
@@ -855,6 +900,9 @@
     <t xml:space="preserve">Pesan WA otomatis saat ada pesanan lunas.</t>
   </si>
   <si>
+    <t xml:space="preserve">Notifikasi_lib::pesanan_dibayar.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Komunikasi &amp; Reputasi</t>
   </si>
   <si>
@@ -903,6 +951,9 @@
     <t xml:space="preserve">Template jawaban satu ketuk.</t>
   </si>
   <si>
+    <t xml:space="preserve">seller/template + tombol template di chat.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Keuangan &amp; Naik Kelas (Pembeda Utama)</t>
   </si>
   <si>
@@ -927,13 +978,7 @@
     <t xml:space="preserve">Penjualan marketplace tercatat otomatis, penjual menambah pengeluaran (bahan, sewa) dengan tombol besar, laporan laba sederhana harian/bulanan.</t>
   </si>
   <si>
-    <t xml:space="preserve">Penjualan offline / kasir mini (POS)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UMKM juga berjualan di warung/pasar, data terpisah</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Catat penjualan langsung, stok tersinkron.</t>
+    <t xml:space="preserve">seller/pembukuan — penjualan marketplace masuk otomatis, kas manual.</t>
   </si>
   <si>
     <t xml:space="preserve">Laporan penjualan &amp; statistik toko</t>
@@ -945,6 +990,9 @@
     <t xml:space="preserve">Grafik omzet, produk terlaris, jam ramai; ekspor Excel/PDF.</t>
   </si>
   <si>
+    <t xml:space="preserve">seller/laporan — grafik omzet, terlaris, jam ramai, ekspor Excel.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Laporan keuangan siap ajukan KUR/pinjaman</t>
   </si>
   <si>
@@ -954,6 +1002,9 @@
     <t xml:space="preserve">Ekspor laporan rapi dari data pembukuan.</t>
   </si>
   <si>
+    <t xml:space="preserve">seller/laporan/kur — laba rugi &amp; arus kas siap cetak.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Voucher &amp; promo toko</t>
   </si>
   <si>
@@ -963,6 +1014,9 @@
     <t xml:space="preserve">Diskon persentase/nominal, voucher pelanggan setia.</t>
   </si>
   <si>
+    <t xml:space="preserve">seller/voucher — persen/nominal, minimal belanja, kuota, khusus pelanggan lama.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Akademi UMKM (pelatihan &amp; pendampingan)</t>
   </si>
   <si>
@@ -972,6 +1026,9 @@
     <t xml:space="preserve">Modul video pendek, kuis, sertifikat, jadwal konsultasi dengan pendamping/mentor.</t>
   </si>
   <si>
+    <t xml:space="preserve">seller/akademi — modul, kuis, sertifikat, jadwal pelatihan.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Skor "Naik Kelas" toko</t>
   </si>
   <si>
@@ -981,6 +1038,9 @@
     <t xml:space="preserve">Level toko (Pemula → Berkembang → Unggul) berdasarkan kelengkapan profil, legalitas, kecepatan respons, rating, dengan saran langkah berikutnya.</t>
   </si>
   <si>
+    <t xml:space="preserve">Naik_kelas_lib — skor 0–100, level Pemula/Berkembang/Unggul, saran langkah berikutnya.</t>
+  </si>
+  <si>
     <t xml:space="preserve">QR code / kartu nama toko digital</t>
   </si>
   <si>
@@ -990,6 +1050,9 @@
     <t xml:space="preserve">QR siap cetak menuju halaman toko.</t>
   </si>
   <si>
+    <t xml:space="preserve">seller/qr — QR &amp; kartu siap cetak (generator QR lokal).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Monitoring</t>
   </si>
   <si>
@@ -1014,6 +1077,9 @@
     <t xml:space="preserve">GMV per periode/wilayah/kategori, pertumbuhan toko, ekspor data.</t>
   </si>
   <si>
+    <t xml:space="preserve">admin/analitik — GMV per periode/wilayah/kategori, ekspor Excel.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Peta sebaran UMKM</t>
   </si>
   <si>
@@ -1023,6 +1089,9 @@
     <t xml:space="preserve">Peta toko per kecamatan beserta tingkat aktivitasnya.</t>
   </si>
   <si>
+    <t xml:space="preserve">admin/peta — peta Leaflet per kecamatan + tingkat aktivitas.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pengguna &amp; Toko</t>
   </si>
   <si>
@@ -1059,6 +1128,9 @@
     <t xml:space="preserve">Antrean verifikasi dokumen, pemberian lencana.</t>
   </si>
   <si>
+    <t xml:space="preserve">admin/verifikasi — antrean dokumen, setujui/tolak, lencana otomatis.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Manajemen pendamping UMKM</t>
   </si>
   <si>
@@ -1068,6 +1140,9 @@
     <t xml:space="preserve">Tetapkan pendamping per toko, catatan kunjungan, progres "naik kelas".</t>
   </si>
   <si>
+    <t xml:space="preserve">admin/pendamping + panel pendamping — catatan kunjungan &amp; progres.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Katalog &amp; Konten</t>
   </si>
   <si>
@@ -1092,6 +1167,9 @@
     <t xml:space="preserve">Daftar produk semua toko, takedown, laporan pengguna.</t>
   </si>
   <si>
+    <t xml:space="preserve">admin/moderasi — turunkan/pulihkan produk, laporan pengguna (Laporkan).</t>
+  </si>
+  <si>
     <t xml:space="preserve">CMS banner &amp; halaman promo</t>
   </si>
   <si>
@@ -1101,6 +1179,9 @@
     <t xml:space="preserve">Atur banner beranda, halaman kampanye ("Pekan Produk Lokal").</t>
   </si>
   <si>
+    <t xml:space="preserve">admin/banner + /promo/{slug}.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Kelola konten Akademi UMKM</t>
   </si>
   <si>
@@ -1110,6 +1191,9 @@
     <t xml:space="preserve">Unggah modul, kuis, jadwal webinar.</t>
   </si>
   <si>
+    <t xml:space="preserve">admin/akademi — modul, soal kuis, jadwal.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Moderasi ulasan &amp; laporan</t>
   </si>
   <si>
@@ -1119,6 +1203,9 @@
     <t xml:space="preserve">Sembunyikan ulasan, tangani laporan.</t>
   </si>
   <si>
+    <t xml:space="preserve">admin/moderasi/ulasan — sembunyikan ulasan, rating dihitung ulang.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Transaksi &amp; Keuangan</t>
   </si>
   <si>
@@ -1179,6 +1266,9 @@
     <t xml:space="preserve">Admin menengahi dengan bukti chat &amp; foto.</t>
   </si>
   <si>
+    <t xml:space="preserve">admin/sengketa — percakapan 3 pihak + keputusan yang membuat refund.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Voucher &amp; subsidi ongkir platform</t>
   </si>
   <si>
@@ -1188,6 +1278,9 @@
     <t xml:space="preserve">Buat voucher platform dengan kuota &amp; anggaran.</t>
   </si>
   <si>
+    <t xml:space="preserve">admin/voucher — kuota &amp; anggaran; subsidi ongkir di Pengaturan.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pengaturan sistem lewat UI</t>
   </si>
   <si>
@@ -1197,6 +1290,9 @@
     <t xml:space="preserve">Halaman pengaturan.</t>
   </si>
   <si>
+    <t xml:space="preserve">admin/pengaturan — komisi, WA, email, ekspedisi, promo, stok.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Komunikasi &amp; Keamanan</t>
   </si>
   <si>
@@ -1209,6 +1305,9 @@
     <t xml:space="preserve">Kirim pengumuman tersegmentasi per wilayah/kategori.</t>
   </si>
   <si>
+    <t xml:space="preserve">admin/broadcast — per wilayah/kategori, banner di panel penjual + WA.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Log audit aktivitas admin</t>
   </si>
   <si>
@@ -1218,7 +1317,7 @@
     <t xml:space="preserve">Riwayat aksi admin.</t>
   </si>
   <si>
-    <t xml:space="preserve">Repo baru punya log status pesanan &amp; callback</t>
+    <t xml:space="preserve">Audit_lib + admin/pengaturan/audit.</t>
   </si>
   <si>
     <t xml:space="preserve">Halaman galat ramah pengguna</t>
@@ -1233,34 +1332,34 @@
     <t xml:space="preserve">Galat.php</t>
   </si>
   <si>
-    <t xml:space="preserve">Tahap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fitur yang Direkomendasikan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quick win (1–2 sprint)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">notifikasi WhatsApp (pembeli &amp; penjual), lupa sandi mandiri, tombol share WA (kodenya sudah ada, tinggal diaktifkan), peringatan stok menipis, mode libur toko, template balasan chat.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pembeda utama (2–4 sprint)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pembukuan sederhana + laporan penjualan, pre-order fleksibel per produk (DP &amp; kalender).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Naik kelas (jangka menengah)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Akademi UMKM, skor "Naik Kelas", bantuan legalitas + lencana verifikasi, laporan siap KUR, manajemen pendamping.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Skala (jangka panjang)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">integrasi agregator ekspedisi, checkout multi-toko, voucher platform, POS offline, PWA.</t>
+    <t xml:space="preserve">Langkah</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Catatan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Langkah 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jalankan migrasi database/24_*.sql sampai database/30_*.sql berurutan (aman diulang; cadangkan dulu).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Langkah 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Isi kunci di Admin &gt; Pengaturan: gerbang WhatsApp (mis. Fonnte), email, dan agregator ekspedisi (mis. Biteship). Tanpa kunci, fitur tetap jalan dengan cara manual (tautan WA, tautan lacak resmi kurir).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Langkah 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dokumen legalitas penjual disimpan di application/dokumen_toko/ (tidak bisa diakses publik). Pastikan server web menolak akses langsung ke /application/.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Langkah 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yang masih bisa dikembangkan: tarif ongkir otomatis dari kurir saat checkout pembeli (kini tarif tetap per wilayah yang diatur penjual; perbandingan tarif kurir tersedia untuk penjual).</t>
   </si>
 </sst>
 </file>
@@ -1503,7 +1602,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="8">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1538,23 +1637,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
           <fgColor rgb="FF006100"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9C0006"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1891,31 +1974,31 @@
         <v>10</v>
       </c>
       <c r="B5" s="5" t="n">
-        <f aca="false">COUNTIF('Daftar Fitur'!$B$2:$B$99,A5)</f>
+        <f aca="false">COUNTIF('Daftar Fitur'!$B$2:$B$97,A5)</f>
         <v>35</v>
       </c>
       <c r="C5" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A5,'Daftar Fitur'!$E$2:$E$99,"Ada")</f>
-        <v>22</v>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$97,A5,'Daftar Fitur'!$E$2:$E$97,"Ada")</f>
+        <v>35</v>
       </c>
       <c r="D5" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A5,'Daftar Fitur'!$E$2:$E$99,"Belum")</f>
-        <v>13</v>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$97,A5,'Daftar Fitur'!$E$2:$E$97,"Belum")</f>
+        <v>0</v>
       </c>
       <c r="E5" s="6" t="n">
         <f aca="false">IF(B5=0,0,C5/B5)</f>
-        <v>0.628571428571429</v>
+        <v>1</v>
       </c>
       <c r="F5" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A5,'Daftar Fitur'!$F$2:$F$99,"Ya")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$97,A5,'Daftar Fitur'!$F$2:$F$97,"Ya")</f>
         <v>4</v>
       </c>
       <c r="G5" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A5,'Daftar Fitur'!$F$2:$F$99,"Ya",'Daftar Fitur'!$E$2:$E$99,"Belum")</f>
-        <v>3</v>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$97,A5,'Daftar Fitur'!$F$2:$F$97,"Ya",'Daftar Fitur'!$E$2:$E$97,"Belum")</f>
+        <v>0</v>
       </c>
       <c r="H5" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A5,'Daftar Fitur'!$G$2:$G$99,"Ya")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$97,A5,'Daftar Fitur'!$G$2:$G$97,"Ya")</f>
         <v>8</v>
       </c>
     </row>
@@ -1924,32 +2007,32 @@
         <v>11</v>
       </c>
       <c r="B6" s="5" t="n">
-        <f aca="false">COUNTIF('Daftar Fitur'!$B$2:$B$99,A6)</f>
-        <v>41</v>
+        <f aca="false">COUNTIF('Daftar Fitur'!$B$2:$B$97,A6)</f>
+        <v>39</v>
       </c>
       <c r="C6" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A6,'Daftar Fitur'!$E$2:$E$99,"Ada")</f>
-        <v>21</v>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$97,A6,'Daftar Fitur'!$E$2:$E$97,"Ada")</f>
+        <v>39</v>
       </c>
       <c r="D6" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A6,'Daftar Fitur'!$E$2:$E$99,"Belum")</f>
-        <v>20</v>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$97,A6,'Daftar Fitur'!$E$2:$E$97,"Belum")</f>
+        <v>0</v>
       </c>
       <c r="E6" s="6" t="n">
         <f aca="false">IF(B6=0,0,C6/B6)</f>
-        <v>0.51219512195122</v>
+        <v>1</v>
       </c>
       <c r="F6" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A6,'Daftar Fitur'!$F$2:$F$99,"Ya")</f>
-        <v>10</v>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$97,A6,'Daftar Fitur'!$F$2:$F$97,"Ya")</f>
+        <v>9</v>
       </c>
       <c r="G6" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A6,'Daftar Fitur'!$F$2:$F$99,"Ya",'Daftar Fitur'!$E$2:$E$99,"Belum")</f>
-        <v>8</v>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$97,A6,'Daftar Fitur'!$F$2:$F$97,"Ya",'Daftar Fitur'!$E$2:$E$97,"Belum")</f>
+        <v>0</v>
       </c>
       <c r="H6" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A6,'Daftar Fitur'!$G$2:$G$99,"Ya")</f>
-        <v>8</v>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$97,A6,'Daftar Fitur'!$G$2:$G$97,"Ya")</f>
+        <v>7</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1957,31 +2040,31 @@
         <v>12</v>
       </c>
       <c r="B7" s="5" t="n">
-        <f aca="false">COUNTIF('Daftar Fitur'!$B$2:$B$99,A7)</f>
+        <f aca="false">COUNTIF('Daftar Fitur'!$B$2:$B$97,A7)</f>
         <v>22</v>
       </c>
       <c r="C7" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A7,'Daftar Fitur'!$E$2:$E$99,"Ada")</f>
-        <v>9</v>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$97,A7,'Daftar Fitur'!$E$2:$E$97,"Ada")</f>
+        <v>22</v>
       </c>
       <c r="D7" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A7,'Daftar Fitur'!$E$2:$E$99,"Belum")</f>
-        <v>13</v>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$97,A7,'Daftar Fitur'!$E$2:$E$97,"Belum")</f>
+        <v>0</v>
       </c>
       <c r="E7" s="6" t="n">
         <f aca="false">IF(B7=0,0,C7/B7)</f>
-        <v>0.409090909090909</v>
+        <v>1</v>
       </c>
       <c r="F7" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A7,'Daftar Fitur'!$F$2:$F$99,"Ya")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$97,A7,'Daftar Fitur'!$F$2:$F$97,"Ya")</f>
         <v>2</v>
       </c>
       <c r="G7" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A7,'Daftar Fitur'!$F$2:$F$99,"Ya",'Daftar Fitur'!$E$2:$E$99,"Belum")</f>
-        <v>2</v>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$97,A7,'Daftar Fitur'!$F$2:$F$97,"Ya",'Daftar Fitur'!$E$2:$E$97,"Belum")</f>
+        <v>0</v>
       </c>
       <c r="H7" s="5" t="n">
-        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$99,A7,'Daftar Fitur'!$G$2:$G$99,"Ya")</f>
+        <f aca="false">COUNTIFS('Daftar Fitur'!$B$2:$B$97,A7,'Daftar Fitur'!$G$2:$G$97,"Ya")</f>
         <v>0</v>
       </c>
     </row>
@@ -1991,31 +2074,31 @@
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">SUM(B5:B7)</f>
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C8" s="8" t="n">
         <f aca="false">SUM(C5:C7)</f>
-        <v>52</v>
+        <v>96</v>
       </c>
       <c r="D8" s="8" t="n">
         <f aca="false">SUM(D5:D7)</f>
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="E8" s="9" t="n">
         <f aca="false">IF(B8=0,0,C8/B8)</f>
-        <v>0.530612244897959</v>
+        <v>1</v>
       </c>
       <c r="F8" s="8" t="n">
         <f aca="false">SUM(F5:F7)</f>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G8" s="8" t="n">
         <f aca="false">SUM(G5:G7)</f>
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="H8" s="8" t="n">
         <f aca="false">SUM(H5:H7)</f>
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2087,7 +2170,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K99"/>
+  <dimension ref="A1:K97"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -2243,7 +2326,7 @@
         <v>49</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F5" s="13"/>
       <c r="G5" s="13" t="s">
@@ -2255,10 +2338,12 @@
       <c r="I5" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="J5" s="14"/>
+      <c r="J5" s="14" t="s">
+        <v>52</v>
+      </c>
       <c r="K5" s="16"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="n">
         <v>5</v>
       </c>
@@ -2269,21 +2354,21 @@
         <v>35</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F6" s="13"/>
       <c r="G6" s="13"/>
       <c r="H6" s="14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I6" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J6" s="14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K6" s="16"/>
     </row>
@@ -2298,7 +2383,7 @@
         <v>35</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E7" s="13" t="s">
         <v>15</v>
@@ -2306,13 +2391,13 @@
       <c r="F7" s="13"/>
       <c r="G7" s="13"/>
       <c r="H7" s="14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I7" s="14" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J7" s="14" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K7" s="16"/>
     </row>
@@ -2324,10 +2409,10 @@
         <v>10</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E8" s="13" t="s">
         <v>15</v>
@@ -2337,13 +2422,13 @@
       </c>
       <c r="G8" s="13"/>
       <c r="H8" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I8" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J8" s="14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K8" s="16"/>
     </row>
@@ -2355,10 +2440,10 @@
         <v>10</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E9" s="13" t="s">
         <v>15</v>
@@ -2366,13 +2451,13 @@
       <c r="F9" s="13"/>
       <c r="G9" s="13"/>
       <c r="H9" s="14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="K9" s="16"/>
     </row>
@@ -2384,10 +2469,10 @@
         <v>10</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E10" s="13" t="s">
         <v>15</v>
@@ -2395,13 +2480,13 @@
       <c r="F10" s="13"/>
       <c r="G10" s="13"/>
       <c r="H10" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I10" s="14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J10" s="14" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K10" s="16"/>
     </row>
@@ -2413,10 +2498,10 @@
         <v>10</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E11" s="13" t="s">
         <v>15</v>
@@ -2424,13 +2509,13 @@
       <c r="F11" s="13"/>
       <c r="G11" s="13"/>
       <c r="H11" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I11" s="14" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J11" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="K11" s="16"/>
     </row>
@@ -2442,10 +2527,10 @@
         <v>10</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E12" s="13" t="s">
         <v>15</v>
@@ -2453,13 +2538,13 @@
       <c r="F12" s="13"/>
       <c r="G12" s="13"/>
       <c r="H12" s="14" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I12" s="14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J12" s="14" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K12" s="16"/>
     </row>
@@ -2471,10 +2556,10 @@
         <v>10</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E13" s="13" t="s">
         <v>15</v>
@@ -2482,17 +2567,17 @@
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
       <c r="H13" s="14" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I13" s="14" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J13" s="14" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K13" s="16"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="n">
         <v>13</v>
       </c>
@@ -2500,23 +2585,25 @@
         <v>10</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F14" s="13"/>
       <c r="G14" s="13"/>
       <c r="H14" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I14" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="J14" s="14"/>
+        <v>88</v>
+      </c>
+      <c r="J14" s="14" t="s">
+        <v>89</v>
+      </c>
       <c r="K14" s="16"/>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2527,26 +2614,28 @@
         <v>10</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F15" s="13"/>
       <c r="G15" s="13"/>
       <c r="H15" s="14" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I15" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="J15" s="14"/>
+        <v>92</v>
+      </c>
+      <c r="J15" s="14" t="s">
+        <v>93</v>
+      </c>
       <c r="K15" s="16"/>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="n">
         <v>15</v>
       </c>
@@ -2554,23 +2643,25 @@
         <v>10</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F16" s="13"/>
       <c r="G16" s="13"/>
       <c r="H16" s="14" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="I16" s="14" t="s">
-        <v>93</v>
-      </c>
-      <c r="J16" s="14"/>
+        <v>96</v>
+      </c>
+      <c r="J16" s="14" t="s">
+        <v>97</v>
+      </c>
       <c r="K16" s="16"/>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2581,28 +2672,30 @@
         <v>10</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F17" s="13" t="s">
         <v>41</v>
       </c>
       <c r="G17" s="13"/>
       <c r="H17" s="14" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="J17" s="14"/>
+        <v>100</v>
+      </c>
+      <c r="J17" s="14" t="s">
+        <v>101</v>
+      </c>
       <c r="K17" s="16"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="n">
         <v>17</v>
       </c>
@@ -2610,26 +2703,26 @@
         <v>10</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F18" s="13"/>
       <c r="G18" s="13" t="s">
         <v>41</v>
       </c>
       <c r="H18" s="14" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="I18" s="14" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="J18" s="14" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="K18" s="16"/>
     </row>
@@ -2641,10 +2734,10 @@
         <v>10</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="E19" s="13" t="s">
         <v>15</v>
@@ -2652,13 +2745,13 @@
       <c r="F19" s="13"/>
       <c r="G19" s="13"/>
       <c r="H19" s="14" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I19" s="14" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="J19" s="14" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="K19" s="16"/>
     </row>
@@ -2670,10 +2763,10 @@
         <v>10</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="E20" s="13" t="s">
         <v>15</v>
@@ -2681,13 +2774,13 @@
       <c r="F20" s="13"/>
       <c r="G20" s="13"/>
       <c r="H20" s="14" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="I20" s="14" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="J20" s="14" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="K20" s="16"/>
     </row>
@@ -2699,10 +2792,10 @@
         <v>10</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="E21" s="13" t="s">
         <v>15</v>
@@ -2710,13 +2803,13 @@
       <c r="F21" s="13"/>
       <c r="G21" s="13"/>
       <c r="H21" s="14" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="I21" s="14" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="J21" s="14" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="K21" s="16"/>
     </row>
@@ -2728,10 +2821,10 @@
         <v>10</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="E22" s="13" t="s">
         <v>15</v>
@@ -2739,13 +2832,13 @@
       <c r="F22" s="13"/>
       <c r="G22" s="13"/>
       <c r="H22" s="14" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="I22" s="14" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="J22" s="14" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="K22" s="16"/>
     </row>
@@ -2757,23 +2850,25 @@
         <v>10</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F23" s="13"/>
       <c r="G23" s="13"/>
       <c r="H23" s="14" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="I23" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="J23" s="14"/>
+        <v>125</v>
+      </c>
+      <c r="J23" s="14" t="s">
+        <v>126</v>
+      </c>
       <c r="K23" s="16"/>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2784,25 +2879,27 @@
         <v>10</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F24" s="13" t="s">
         <v>41</v>
       </c>
       <c r="G24" s="13"/>
       <c r="H24" s="14" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="I24" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="J24" s="14"/>
+        <v>129</v>
+      </c>
+      <c r="J24" s="14" t="s">
+        <v>130</v>
+      </c>
       <c r="K24" s="16"/>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2813,26 +2910,26 @@
         <v>10</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F25" s="13" t="s">
         <v>41</v>
       </c>
       <c r="G25" s="13"/>
       <c r="H25" s="14" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="I25" s="14" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="J25" s="14" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="K25" s="16"/>
     </row>
@@ -2844,10 +2941,10 @@
         <v>10</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="E26" s="13" t="s">
         <v>15</v>
@@ -2855,13 +2952,13 @@
       <c r="F26" s="13"/>
       <c r="G26" s="13"/>
       <c r="H26" s="14" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="I26" s="14" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="J26" s="14" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="K26" s="16"/>
     </row>
@@ -2873,10 +2970,10 @@
         <v>10</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="E27" s="13" t="s">
         <v>15</v>
@@ -2884,13 +2981,13 @@
       <c r="F27" s="13"/>
       <c r="G27" s="13"/>
       <c r="H27" s="14" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="I27" s="14" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="J27" s="14" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="K27" s="16"/>
     </row>
@@ -2902,10 +2999,10 @@
         <v>10</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="E28" s="13" t="s">
         <v>15</v>
@@ -2913,13 +3010,13 @@
       <c r="F28" s="13"/>
       <c r="G28" s="13"/>
       <c r="H28" s="14" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="I28" s="14" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="J28" s="14" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="K28" s="16"/>
     </row>
@@ -2931,10 +3028,10 @@
         <v>10</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="E29" s="13" t="s">
         <v>15</v>
@@ -2942,13 +3039,13 @@
       <c r="F29" s="13"/>
       <c r="G29" s="13"/>
       <c r="H29" s="14" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="I29" s="14" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="J29" s="14" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="K29" s="16"/>
     </row>
@@ -2960,10 +3057,10 @@
         <v>10</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="E30" s="13" t="s">
         <v>15</v>
@@ -2971,13 +3068,13 @@
       <c r="F30" s="13"/>
       <c r="G30" s="13"/>
       <c r="H30" s="14" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="I30" s="14" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="J30" s="14" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="K30" s="16"/>
     </row>
@@ -2989,10 +3086,10 @@
         <v>10</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="E31" s="13" t="s">
         <v>15</v>
@@ -3000,13 +3097,13 @@
       <c r="F31" s="13"/>
       <c r="G31" s="13"/>
       <c r="H31" s="14" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="I31" s="14" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="J31" s="14" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="K31" s="16"/>
     </row>
@@ -3018,10 +3115,10 @@
         <v>10</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="E32" s="13" t="s">
         <v>15</v>
@@ -3029,17 +3126,17 @@
       <c r="F32" s="13"/>
       <c r="G32" s="13"/>
       <c r="H32" s="14" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="I32" s="14" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="J32" s="14" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="K32" s="16"/>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="n">
         <v>32</v>
       </c>
@@ -3047,25 +3144,27 @@
         <v>10</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F33" s="13"/>
       <c r="G33" s="13" t="s">
         <v>41</v>
       </c>
       <c r="H33" s="14" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="I33" s="14" t="s">
-        <v>159</v>
-      </c>
-      <c r="J33" s="14"/>
+        <v>166</v>
+      </c>
+      <c r="J33" s="14" t="s">
+        <v>167</v>
+      </c>
       <c r="K33" s="16"/>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3076,10 +3175,10 @@
         <v>10</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="E34" s="13" t="s">
         <v>15</v>
@@ -3089,13 +3188,13 @@
         <v>41</v>
       </c>
       <c r="H34" s="14" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="I34" s="14" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="J34" s="14" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="K34" s="16"/>
     </row>
@@ -3107,25 +3206,27 @@
         <v>10</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F35" s="13"/>
       <c r="G35" s="13" t="s">
         <v>41</v>
       </c>
       <c r="H35" s="14" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="I35" s="14" t="s">
-        <v>167</v>
-      </c>
-      <c r="J35" s="14"/>
+        <v>175</v>
+      </c>
+      <c r="J35" s="14" t="s">
+        <v>176</v>
+      </c>
       <c r="K35" s="16"/>
     </row>
     <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3136,25 +3237,27 @@
         <v>10</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F36" s="13"/>
       <c r="G36" s="13" t="s">
         <v>41</v>
       </c>
       <c r="H36" s="14" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="I36" s="14" t="s">
-        <v>170</v>
-      </c>
-      <c r="J36" s="14"/>
+        <v>179</v>
+      </c>
+      <c r="J36" s="14" t="s">
+        <v>180</v>
+      </c>
       <c r="K36" s="16"/>
     </row>
     <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3165,10 +3268,10 @@
         <v>11</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="E37" s="13" t="s">
         <v>15</v>
@@ -3178,13 +3281,13 @@
         <v>41</v>
       </c>
       <c r="H37" s="14" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="I37" s="14" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
       <c r="J37" s="14" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="K37" s="16"/>
     </row>
@@ -3196,10 +3299,10 @@
         <v>11</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="D38" s="15" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>15</v>
@@ -3207,13 +3310,13 @@
       <c r="F38" s="13"/>
       <c r="G38" s="13"/>
       <c r="H38" s="14" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="I38" s="14" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
       <c r="J38" s="14" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="K38" s="16"/>
     </row>
@@ -3225,10 +3328,10 @@
         <v>11</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="D39" s="15" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="E39" s="13" t="s">
         <v>15</v>
@@ -3236,13 +3339,13 @@
       <c r="F39" s="13"/>
       <c r="G39" s="13"/>
       <c r="H39" s="14" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
       <c r="I39" s="14" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="J39" s="14" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="K39" s="16"/>
     </row>
@@ -3254,25 +3357,27 @@
         <v>11</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="D40" s="15" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F40" s="13"/>
       <c r="G40" s="13" t="s">
         <v>41</v>
       </c>
       <c r="H40" s="14" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
       <c r="I40" s="14" t="s">
-        <v>186</v>
-      </c>
-      <c r="J40" s="14"/>
+        <v>196</v>
+      </c>
+      <c r="J40" s="14" t="s">
+        <v>197</v>
+      </c>
       <c r="K40" s="16"/>
     </row>
     <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3283,25 +3388,27 @@
         <v>11</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="D41" s="15" t="s">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="E41" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F41" s="13" t="s">
         <v>41</v>
       </c>
       <c r="G41" s="13"/>
       <c r="H41" s="14" t="s">
-        <v>188</v>
+        <v>199</v>
       </c>
       <c r="I41" s="14" t="s">
-        <v>189</v>
-      </c>
-      <c r="J41" s="14"/>
+        <v>200</v>
+      </c>
+      <c r="J41" s="14" t="s">
+        <v>201</v>
+      </c>
       <c r="K41" s="16"/>
     </row>
     <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3312,24 +3419,24 @@
         <v>11</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="D42" s="15" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F42" s="13"/>
       <c r="G42" s="13"/>
       <c r="H42" s="14" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="I42" s="14" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="J42" s="14" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="K42" s="16"/>
     </row>
@@ -3341,10 +3448,10 @@
         <v>11</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="D43" s="15" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="E43" s="13" t="s">
         <v>15</v>
@@ -3352,13 +3459,13 @@
       <c r="F43" s="13"/>
       <c r="G43" s="13"/>
       <c r="H43" s="14" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
       <c r="I43" s="14" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="J43" s="14" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="K43" s="16"/>
     </row>
@@ -3370,10 +3477,10 @@
         <v>11</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="D44" s="15" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="E44" s="13" t="s">
         <v>15</v>
@@ -3381,13 +3488,13 @@
       <c r="F44" s="13"/>
       <c r="G44" s="13"/>
       <c r="H44" s="14" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="I44" s="14" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="J44" s="14" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="K44" s="16"/>
     </row>
@@ -3399,10 +3506,10 @@
         <v>11</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="D45" s="15" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="E45" s="13" t="s">
         <v>15</v>
@@ -3410,13 +3517,13 @@
       <c r="F45" s="13"/>
       <c r="G45" s="13"/>
       <c r="H45" s="14" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="I45" s="14" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="J45" s="14" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="K45" s="16"/>
     </row>
@@ -3428,10 +3535,10 @@
         <v>11</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="D46" s="15" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="E46" s="13" t="s">
         <v>15</v>
@@ -3439,13 +3546,13 @@
       <c r="F46" s="13"/>
       <c r="G46" s="13"/>
       <c r="H46" s="14" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="I46" s="14" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="J46" s="14" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="K46" s="16"/>
     </row>
@@ -3457,10 +3564,10 @@
         <v>11</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="D47" s="15" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="E47" s="13" t="s">
         <v>15</v>
@@ -3472,13 +3579,13 @@
         <v>41</v>
       </c>
       <c r="H47" s="14" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="I47" s="14" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="J47" s="14" t="s">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="K47" s="16"/>
     </row>
@@ -3490,10 +3597,10 @@
         <v>11</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="D48" s="15" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="E48" s="13" t="s">
         <v>15</v>
@@ -3501,13 +3608,13 @@
       <c r="F48" s="13"/>
       <c r="G48" s="13"/>
       <c r="H48" s="14" t="s">
-        <v>216</v>
+        <v>228</v>
       </c>
       <c r="I48" s="14" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
       <c r="J48" s="14" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="K48" s="16"/>
     </row>
@@ -3519,25 +3626,25 @@
         <v>11</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="D49" s="15" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="E49" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F49" s="13"/>
-      <c r="G49" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="G49" s="13"/>
       <c r="H49" s="14" t="s">
-        <v>220</v>
+        <v>232</v>
       </c>
       <c r="I49" s="14" t="s">
-        <v>221</v>
-      </c>
-      <c r="J49" s="14"/>
+        <v>233</v>
+      </c>
+      <c r="J49" s="14" t="s">
+        <v>234</v>
+      </c>
       <c r="K49" s="16"/>
     </row>
     <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3548,23 +3655,25 @@
         <v>11</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="D50" s="15" t="s">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="E50" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F50" s="13"/>
       <c r="G50" s="13"/>
       <c r="H50" s="14" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="I50" s="14" t="s">
-        <v>224</v>
-      </c>
-      <c r="J50" s="14"/>
+        <v>237</v>
+      </c>
+      <c r="J50" s="14" t="s">
+        <v>238</v>
+      </c>
       <c r="K50" s="16"/>
     </row>
     <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3575,23 +3684,27 @@
         <v>11</v>
       </c>
       <c r="C51" s="14" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="D51" s="15" t="s">
-        <v>225</v>
+        <v>239</v>
       </c>
       <c r="E51" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F51" s="13"/>
+        <v>15</v>
+      </c>
+      <c r="F51" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="G51" s="13"/>
       <c r="H51" s="14" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="I51" s="14" t="s">
-        <v>227</v>
-      </c>
-      <c r="J51" s="14"/>
+        <v>241</v>
+      </c>
+      <c r="J51" s="14" t="s">
+        <v>242</v>
+      </c>
       <c r="K51" s="16"/>
     </row>
     <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3602,25 +3715,27 @@
         <v>11</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="D52" s="15" t="s">
-        <v>228</v>
+        <v>243</v>
       </c>
       <c r="E52" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F52" s="13" t="s">
         <v>41</v>
       </c>
       <c r="G52" s="13"/>
       <c r="H52" s="14" t="s">
-        <v>229</v>
+        <v>244</v>
       </c>
       <c r="I52" s="14" t="s">
-        <v>230</v>
-      </c>
-      <c r="J52" s="14"/>
+        <v>245</v>
+      </c>
+      <c r="J52" s="14" t="s">
+        <v>246</v>
+      </c>
       <c r="K52" s="16"/>
     </row>
     <row r="53" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3631,25 +3746,27 @@
         <v>11</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>194</v>
+        <v>247</v>
       </c>
       <c r="D53" s="15" t="s">
-        <v>231</v>
+        <v>248</v>
       </c>
       <c r="E53" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F53" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F53" s="13"/>
+      <c r="G53" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="G53" s="13"/>
       <c r="H53" s="14" t="s">
-        <v>232</v>
+        <v>249</v>
       </c>
       <c r="I53" s="14" t="s">
-        <v>233</v>
-      </c>
-      <c r="J53" s="14"/>
+        <v>250</v>
+      </c>
+      <c r="J53" s="14" t="s">
+        <v>251</v>
+      </c>
       <c r="K53" s="16"/>
     </row>
     <row r="54" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3660,26 +3777,24 @@
         <v>11</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="D54" s="15" t="s">
-        <v>235</v>
+        <v>252</v>
       </c>
       <c r="E54" s="13" t="s">
         <v>15</v>
       </c>
       <c r="F54" s="13"/>
-      <c r="G54" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="G54" s="13"/>
       <c r="H54" s="14" t="s">
-        <v>236</v>
+        <v>253</v>
       </c>
       <c r="I54" s="14" t="s">
-        <v>237</v>
+        <v>254</v>
       </c>
       <c r="J54" s="14" t="s">
-        <v>238</v>
+        <v>255</v>
       </c>
       <c r="K54" s="16"/>
     </row>
@@ -3691,24 +3806,26 @@
         <v>11</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="D55" s="15" t="s">
-        <v>239</v>
+        <v>256</v>
       </c>
       <c r="E55" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="F55" s="13"/>
+      <c r="F55" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="G55" s="13"/>
       <c r="H55" s="14" t="s">
-        <v>240</v>
+        <v>257</v>
       </c>
       <c r="I55" s="14" t="s">
-        <v>241</v>
+        <v>258</v>
       </c>
       <c r="J55" s="14" t="s">
-        <v>242</v>
+        <v>259</v>
       </c>
       <c r="K55" s="16"/>
     </row>
@@ -3720,26 +3837,24 @@
         <v>11</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="D56" s="15" t="s">
-        <v>243</v>
+        <v>260</v>
       </c>
       <c r="E56" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="F56" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="F56" s="13"/>
       <c r="G56" s="13"/>
       <c r="H56" s="14" t="s">
-        <v>244</v>
+        <v>261</v>
       </c>
       <c r="I56" s="14" t="s">
-        <v>245</v>
+        <v>262</v>
       </c>
       <c r="J56" s="14" t="s">
-        <v>246</v>
+        <v>263</v>
       </c>
       <c r="K56" s="16"/>
     </row>
@@ -3751,10 +3866,10 @@
         <v>11</v>
       </c>
       <c r="C57" s="14" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="D57" s="15" t="s">
-        <v>247</v>
+        <v>264</v>
       </c>
       <c r="E57" s="13" t="s">
         <v>15</v>
@@ -3762,13 +3877,13 @@
       <c r="F57" s="13"/>
       <c r="G57" s="13"/>
       <c r="H57" s="14" t="s">
-        <v>248</v>
+        <v>265</v>
       </c>
       <c r="I57" s="14" t="s">
-        <v>249</v>
+        <v>266</v>
       </c>
       <c r="J57" s="14" t="s">
-        <v>250</v>
+        <v>267</v>
       </c>
       <c r="K57" s="16"/>
     </row>
@@ -3780,10 +3895,10 @@
         <v>11</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="D58" s="15" t="s">
-        <v>251</v>
+        <v>268</v>
       </c>
       <c r="E58" s="13" t="s">
         <v>15</v>
@@ -3791,13 +3906,13 @@
       <c r="F58" s="13"/>
       <c r="G58" s="13"/>
       <c r="H58" s="14" t="s">
-        <v>252</v>
+        <v>269</v>
       </c>
       <c r="I58" s="14" t="s">
-        <v>253</v>
+        <v>270</v>
       </c>
       <c r="J58" s="14" t="s">
-        <v>254</v>
+        <v>271</v>
       </c>
       <c r="K58" s="16"/>
     </row>
@@ -3809,10 +3924,10 @@
         <v>11</v>
       </c>
       <c r="C59" s="14" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="D59" s="15" t="s">
-        <v>255</v>
+        <v>272</v>
       </c>
       <c r="E59" s="13" t="s">
         <v>15</v>
@@ -3820,13 +3935,13 @@
       <c r="F59" s="13"/>
       <c r="G59" s="13"/>
       <c r="H59" s="14" t="s">
-        <v>256</v>
+        <v>273</v>
       </c>
       <c r="I59" s="14" t="s">
-        <v>257</v>
+        <v>274</v>
       </c>
       <c r="J59" s="14" t="s">
-        <v>258</v>
+        <v>275</v>
       </c>
       <c r="K59" s="16"/>
     </row>
@@ -3838,10 +3953,10 @@
         <v>11</v>
       </c>
       <c r="C60" s="14" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="D60" s="15" t="s">
-        <v>259</v>
+        <v>276</v>
       </c>
       <c r="E60" s="13" t="s">
         <v>15</v>
@@ -3849,17 +3964,17 @@
       <c r="F60" s="13"/>
       <c r="G60" s="13"/>
       <c r="H60" s="14" t="s">
-        <v>260</v>
+        <v>277</v>
       </c>
       <c r="I60" s="14" t="s">
-        <v>261</v>
+        <v>278</v>
       </c>
       <c r="J60" s="14" t="s">
-        <v>262</v>
+        <v>279</v>
       </c>
       <c r="K60" s="16"/>
     </row>
-    <row r="61" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="13" t="n">
         <v>60</v>
       </c>
@@ -3867,10 +3982,10 @@
         <v>11</v>
       </c>
       <c r="C61" s="14" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="D61" s="15" t="s">
-        <v>263</v>
+        <v>280</v>
       </c>
       <c r="E61" s="13" t="s">
         <v>15</v>
@@ -3878,13 +3993,13 @@
       <c r="F61" s="13"/>
       <c r="G61" s="13"/>
       <c r="H61" s="14" t="s">
-        <v>264</v>
+        <v>281</v>
       </c>
       <c r="I61" s="14" t="s">
-        <v>265</v>
+        <v>282</v>
       </c>
       <c r="J61" s="14" t="s">
-        <v>266</v>
+        <v>283</v>
       </c>
       <c r="K61" s="16"/>
     </row>
@@ -3896,23 +4011,27 @@
         <v>11</v>
       </c>
       <c r="C62" s="14" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="D62" s="15" t="s">
-        <v>267</v>
+        <v>284</v>
       </c>
       <c r="E62" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F62" s="13"/>
-      <c r="G62" s="13"/>
+      <c r="G62" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="H62" s="14" t="s">
-        <v>268</v>
+        <v>285</v>
       </c>
       <c r="I62" s="14" t="s">
-        <v>269</v>
-      </c>
-      <c r="J62" s="14"/>
+        <v>286</v>
+      </c>
+      <c r="J62" s="14" t="s">
+        <v>287</v>
+      </c>
       <c r="K62" s="16"/>
     </row>
     <row r="63" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3923,25 +4042,25 @@
         <v>11</v>
       </c>
       <c r="C63" s="14" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="D63" s="15" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
       <c r="E63" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F63" s="13"/>
-      <c r="G63" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="G63" s="13"/>
       <c r="H63" s="14" t="s">
-        <v>271</v>
+        <v>289</v>
       </c>
       <c r="I63" s="14" t="s">
-        <v>272</v>
-      </c>
-      <c r="J63" s="14"/>
+        <v>290</v>
+      </c>
+      <c r="J63" s="14" t="s">
+        <v>291</v>
+      </c>
       <c r="K63" s="16"/>
     </row>
     <row r="64" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3952,23 +4071,25 @@
         <v>11</v>
       </c>
       <c r="C64" s="14" t="s">
-        <v>234</v>
+        <v>292</v>
       </c>
       <c r="D64" s="15" t="s">
-        <v>273</v>
+        <v>293</v>
       </c>
       <c r="E64" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F64" s="13"/>
       <c r="G64" s="13"/>
       <c r="H64" s="14" t="s">
-        <v>274</v>
+        <v>294</v>
       </c>
       <c r="I64" s="14" t="s">
-        <v>275</v>
-      </c>
-      <c r="J64" s="14"/>
+        <v>295</v>
+      </c>
+      <c r="J64" s="14" t="s">
+        <v>296</v>
+      </c>
       <c r="K64" s="16"/>
     </row>
     <row r="65" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3979,10 +4100,10 @@
         <v>11</v>
       </c>
       <c r="C65" s="14" t="s">
-        <v>276</v>
+        <v>292</v>
       </c>
       <c r="D65" s="15" t="s">
-        <v>277</v>
+        <v>297</v>
       </c>
       <c r="E65" s="13" t="s">
         <v>15</v>
@@ -3990,13 +4111,13 @@
       <c r="F65" s="13"/>
       <c r="G65" s="13"/>
       <c r="H65" s="14" t="s">
-        <v>278</v>
+        <v>298</v>
       </c>
       <c r="I65" s="14" t="s">
-        <v>279</v>
+        <v>299</v>
       </c>
       <c r="J65" s="14" t="s">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="K65" s="16"/>
     </row>
@@ -4008,10 +4129,10 @@
         <v>11</v>
       </c>
       <c r="C66" s="14" t="s">
-        <v>276</v>
+        <v>292</v>
       </c>
       <c r="D66" s="15" t="s">
-        <v>281</v>
+        <v>301</v>
       </c>
       <c r="E66" s="13" t="s">
         <v>15</v>
@@ -4019,13 +4140,13 @@
       <c r="F66" s="13"/>
       <c r="G66" s="13"/>
       <c r="H66" s="14" t="s">
-        <v>282</v>
+        <v>302</v>
       </c>
       <c r="I66" s="14" t="s">
-        <v>283</v>
+        <v>303</v>
       </c>
       <c r="J66" s="14" t="s">
-        <v>284</v>
+        <v>304</v>
       </c>
       <c r="K66" s="16"/>
     </row>
@@ -4037,24 +4158,26 @@
         <v>11</v>
       </c>
       <c r="C67" s="14" t="s">
-        <v>276</v>
+        <v>292</v>
       </c>
       <c r="D67" s="15" t="s">
-        <v>285</v>
+        <v>305</v>
       </c>
       <c r="E67" s="13" t="s">
         <v>15</v>
       </c>
       <c r="F67" s="13"/>
-      <c r="G67" s="13"/>
+      <c r="G67" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="H67" s="14" t="s">
-        <v>286</v>
+        <v>306</v>
       </c>
       <c r="I67" s="14" t="s">
-        <v>287</v>
+        <v>307</v>
       </c>
       <c r="J67" s="14" t="s">
-        <v>288</v>
+        <v>308</v>
       </c>
       <c r="K67" s="16"/>
     </row>
@@ -4066,28 +4189,28 @@
         <v>11</v>
       </c>
       <c r="C68" s="14" t="s">
-        <v>276</v>
+        <v>309</v>
       </c>
       <c r="D68" s="15" t="s">
-        <v>289</v>
+        <v>310</v>
       </c>
       <c r="E68" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F68" s="13"/>
-      <c r="G68" s="13" t="s">
-        <v>41</v>
-      </c>
+      <c r="G68" s="13"/>
       <c r="H68" s="14" t="s">
-        <v>290</v>
+        <v>311</v>
       </c>
       <c r="I68" s="14" t="s">
-        <v>291</v>
-      </c>
-      <c r="J68" s="14"/>
+        <v>312</v>
+      </c>
+      <c r="J68" s="14" t="s">
+        <v>313</v>
+      </c>
       <c r="K68" s="16"/>
     </row>
-    <row r="69" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="13" t="n">
         <v>68</v>
       </c>
@@ -4095,28 +4218,32 @@
         <v>11</v>
       </c>
       <c r="C69" s="14" t="s">
-        <v>292</v>
+        <v>309</v>
       </c>
       <c r="D69" s="15" t="s">
-        <v>293</v>
+        <v>314</v>
       </c>
       <c r="E69" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="F69" s="13"/>
-      <c r="G69" s="13"/>
+      <c r="F69" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="G69" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="H69" s="14" t="s">
-        <v>294</v>
+        <v>315</v>
       </c>
       <c r="I69" s="14" t="s">
-        <v>295</v>
+        <v>316</v>
       </c>
       <c r="J69" s="14" t="s">
-        <v>296</v>
+        <v>317</v>
       </c>
       <c r="K69" s="16"/>
     </row>
-    <row r="70" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="13" t="n">
         <v>69</v>
       </c>
@@ -4124,27 +4251,25 @@
         <v>11</v>
       </c>
       <c r="C70" s="14" t="s">
-        <v>292</v>
+        <v>309</v>
       </c>
       <c r="D70" s="15" t="s">
-        <v>297</v>
+        <v>318</v>
       </c>
       <c r="E70" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F70" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="G70" s="13" t="s">
-        <v>41</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="F70" s="13"/>
+      <c r="G70" s="13"/>
       <c r="H70" s="14" t="s">
-        <v>298</v>
+        <v>319</v>
       </c>
       <c r="I70" s="14" t="s">
-        <v>299</v>
-      </c>
-      <c r="J70" s="14"/>
+        <v>320</v>
+      </c>
+      <c r="J70" s="14" t="s">
+        <v>321</v>
+      </c>
       <c r="K70" s="16"/>
     </row>
     <row r="71" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4155,25 +4280,27 @@
         <v>11</v>
       </c>
       <c r="C71" s="14" t="s">
-        <v>292</v>
+        <v>309</v>
       </c>
       <c r="D71" s="15" t="s">
-        <v>300</v>
+        <v>322</v>
       </c>
       <c r="E71" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F71" s="13" t="s">
         <v>41</v>
       </c>
       <c r="G71" s="13"/>
       <c r="H71" s="14" t="s">
-        <v>301</v>
+        <v>323</v>
       </c>
       <c r="I71" s="14" t="s">
-        <v>302</v>
-      </c>
-      <c r="J71" s="14"/>
+        <v>324</v>
+      </c>
+      <c r="J71" s="14" t="s">
+        <v>325</v>
+      </c>
       <c r="K71" s="16"/>
     </row>
     <row r="72" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4184,23 +4311,25 @@
         <v>11</v>
       </c>
       <c r="C72" s="14" t="s">
-        <v>292</v>
+        <v>309</v>
       </c>
       <c r="D72" s="15" t="s">
-        <v>303</v>
+        <v>326</v>
       </c>
       <c r="E72" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F72" s="13"/>
       <c r="G72" s="13"/>
       <c r="H72" s="14" t="s">
-        <v>304</v>
+        <v>327</v>
       </c>
       <c r="I72" s="14" t="s">
-        <v>305</v>
-      </c>
-      <c r="J72" s="14"/>
+        <v>328</v>
+      </c>
+      <c r="J72" s="14" t="s">
+        <v>329</v>
+      </c>
       <c r="K72" s="16"/>
     </row>
     <row r="73" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4211,28 +4340,30 @@
         <v>11</v>
       </c>
       <c r="C73" s="14" t="s">
-        <v>292</v>
+        <v>309</v>
       </c>
       <c r="D73" s="15" t="s">
-        <v>306</v>
+        <v>330</v>
       </c>
       <c r="E73" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F73" s="13" t="s">
         <v>41</v>
       </c>
       <c r="G73" s="13"/>
       <c r="H73" s="14" t="s">
-        <v>307</v>
+        <v>331</v>
       </c>
       <c r="I73" s="14" t="s">
-        <v>308</v>
-      </c>
-      <c r="J73" s="14"/>
+        <v>332</v>
+      </c>
+      <c r="J73" s="14" t="s">
+        <v>333</v>
+      </c>
       <c r="K73" s="16"/>
     </row>
-    <row r="74" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="13" t="n">
         <v>73</v>
       </c>
@@ -4240,23 +4371,27 @@
         <v>11</v>
       </c>
       <c r="C74" s="14" t="s">
-        <v>292</v>
+        <v>309</v>
       </c>
       <c r="D74" s="15" t="s">
-        <v>309</v>
+        <v>334</v>
       </c>
       <c r="E74" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F74" s="13"/>
+        <v>15</v>
+      </c>
+      <c r="F74" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="G74" s="13"/>
       <c r="H74" s="14" t="s">
-        <v>310</v>
+        <v>335</v>
       </c>
       <c r="I74" s="14" t="s">
-        <v>311</v>
-      </c>
-      <c r="J74" s="14"/>
+        <v>336</v>
+      </c>
+      <c r="J74" s="14" t="s">
+        <v>337</v>
+      </c>
       <c r="K74" s="16"/>
     </row>
     <row r="75" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4267,54 +4402,54 @@
         <v>11</v>
       </c>
       <c r="C75" s="14" t="s">
-        <v>292</v>
+        <v>309</v>
       </c>
       <c r="D75" s="15" t="s">
-        <v>312</v>
+        <v>338</v>
       </c>
       <c r="E75" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F75" s="13" t="s">
-        <v>41</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="F75" s="13"/>
       <c r="G75" s="13"/>
       <c r="H75" s="14" t="s">
-        <v>313</v>
+        <v>339</v>
       </c>
       <c r="I75" s="14" t="s">
-        <v>314</v>
-      </c>
-      <c r="J75" s="14"/>
+        <v>340</v>
+      </c>
+      <c r="J75" s="14" t="s">
+        <v>341</v>
+      </c>
       <c r="K75" s="16"/>
     </row>
-    <row r="76" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="13" t="n">
         <v>75</v>
       </c>
       <c r="B76" s="14" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C76" s="14" t="s">
-        <v>292</v>
+        <v>342</v>
       </c>
       <c r="D76" s="15" t="s">
-        <v>315</v>
+        <v>343</v>
       </c>
       <c r="E76" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F76" s="13" t="s">
-        <v>41</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="F76" s="13"/>
       <c r="G76" s="13"/>
       <c r="H76" s="14" t="s">
-        <v>316</v>
+        <v>344</v>
       </c>
       <c r="I76" s="14" t="s">
-        <v>317</v>
-      </c>
-      <c r="J76" s="14"/>
+        <v>345</v>
+      </c>
+      <c r="J76" s="14" t="s">
+        <v>346</v>
+      </c>
       <c r="K76" s="16"/>
     </row>
     <row r="77" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4322,26 +4457,28 @@
         <v>76</v>
       </c>
       <c r="B77" s="14" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C77" s="14" t="s">
-        <v>292</v>
+        <v>342</v>
       </c>
       <c r="D77" s="15" t="s">
-        <v>318</v>
+        <v>347</v>
       </c>
       <c r="E77" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F77" s="13"/>
       <c r="G77" s="13"/>
       <c r="H77" s="14" t="s">
-        <v>319</v>
+        <v>348</v>
       </c>
       <c r="I77" s="14" t="s">
-        <v>320</v>
-      </c>
-      <c r="J77" s="14"/>
+        <v>349</v>
+      </c>
+      <c r="J77" s="14" t="s">
+        <v>350</v>
+      </c>
       <c r="K77" s="16"/>
     </row>
     <row r="78" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4352,24 +4489,26 @@
         <v>12</v>
       </c>
       <c r="C78" s="14" t="s">
-        <v>321</v>
+        <v>342</v>
       </c>
       <c r="D78" s="15" t="s">
-        <v>322</v>
+        <v>351</v>
       </c>
       <c r="E78" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="F78" s="13"/>
+      <c r="F78" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="G78" s="13"/>
       <c r="H78" s="14" t="s">
-        <v>323</v>
+        <v>352</v>
       </c>
       <c r="I78" s="14" t="s">
-        <v>324</v>
+        <v>353</v>
       </c>
       <c r="J78" s="14" t="s">
-        <v>325</v>
+        <v>354</v>
       </c>
       <c r="K78" s="16"/>
     </row>
@@ -4381,23 +4520,25 @@
         <v>12</v>
       </c>
       <c r="C79" s="14" t="s">
-        <v>321</v>
+        <v>355</v>
       </c>
       <c r="D79" s="15" t="s">
-        <v>326</v>
+        <v>356</v>
       </c>
       <c r="E79" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F79" s="13"/>
       <c r="G79" s="13"/>
       <c r="H79" s="14" t="s">
-        <v>327</v>
+        <v>357</v>
       </c>
       <c r="I79" s="14" t="s">
-        <v>328</v>
-      </c>
-      <c r="J79" s="14"/>
+        <v>358</v>
+      </c>
+      <c r="J79" s="14" t="s">
+        <v>359</v>
+      </c>
       <c r="K79" s="16"/>
     </row>
     <row r="80" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4408,25 +4549,25 @@
         <v>12</v>
       </c>
       <c r="C80" s="14" t="s">
-        <v>321</v>
+        <v>355</v>
       </c>
       <c r="D80" s="15" t="s">
-        <v>329</v>
+        <v>360</v>
       </c>
       <c r="E80" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F80" s="13" t="s">
-        <v>41</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="F80" s="13"/>
       <c r="G80" s="13"/>
       <c r="H80" s="14" t="s">
-        <v>330</v>
+        <v>361</v>
       </c>
       <c r="I80" s="14" t="s">
-        <v>331</v>
-      </c>
-      <c r="J80" s="14"/>
+        <v>362</v>
+      </c>
+      <c r="J80" s="14" t="s">
+        <v>363</v>
+      </c>
       <c r="K80" s="16"/>
     </row>
     <row r="81" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4437,10 +4578,10 @@
         <v>12</v>
       </c>
       <c r="C81" s="14" t="s">
-        <v>332</v>
+        <v>355</v>
       </c>
       <c r="D81" s="15" t="s">
-        <v>333</v>
+        <v>364</v>
       </c>
       <c r="E81" s="13" t="s">
         <v>15</v>
@@ -4448,13 +4589,13 @@
       <c r="F81" s="13"/>
       <c r="G81" s="13"/>
       <c r="H81" s="14" t="s">
-        <v>334</v>
+        <v>365</v>
       </c>
       <c r="I81" s="14" t="s">
-        <v>335</v>
+        <v>366</v>
       </c>
       <c r="J81" s="14" t="s">
-        <v>336</v>
+        <v>367</v>
       </c>
       <c r="K81" s="16"/>
     </row>
@@ -4466,24 +4607,26 @@
         <v>12</v>
       </c>
       <c r="C82" s="14" t="s">
-        <v>332</v>
+        <v>355</v>
       </c>
       <c r="D82" s="15" t="s">
-        <v>337</v>
+        <v>368</v>
       </c>
       <c r="E82" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="F82" s="13"/>
+      <c r="F82" s="13" t="s">
+        <v>41</v>
+      </c>
       <c r="G82" s="13"/>
       <c r="H82" s="14" t="s">
-        <v>338</v>
+        <v>369</v>
       </c>
       <c r="I82" s="14" t="s">
-        <v>339</v>
+        <v>370</v>
       </c>
       <c r="J82" s="14" t="s">
-        <v>340</v>
+        <v>371</v>
       </c>
       <c r="K82" s="16"/>
     </row>
@@ -4495,23 +4638,25 @@
         <v>12</v>
       </c>
       <c r="C83" s="14" t="s">
-        <v>332</v>
+        <v>372</v>
       </c>
       <c r="D83" s="15" t="s">
-        <v>341</v>
+        <v>373</v>
       </c>
       <c r="E83" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F83" s="13"/>
       <c r="G83" s="13"/>
       <c r="H83" s="14" t="s">
-        <v>342</v>
+        <v>374</v>
       </c>
       <c r="I83" s="14" t="s">
-        <v>343</v>
-      </c>
-      <c r="J83" s="14"/>
+        <v>375</v>
+      </c>
+      <c r="J83" s="14" t="s">
+        <v>376</v>
+      </c>
       <c r="K83" s="16"/>
     </row>
     <row r="84" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4522,25 +4667,25 @@
         <v>12</v>
       </c>
       <c r="C84" s="14" t="s">
-        <v>332</v>
+        <v>372</v>
       </c>
       <c r="D84" s="15" t="s">
-        <v>344</v>
+        <v>377</v>
       </c>
       <c r="E84" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F84" s="13" t="s">
-        <v>41</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="F84" s="13"/>
       <c r="G84" s="13"/>
       <c r="H84" s="14" t="s">
-        <v>345</v>
+        <v>378</v>
       </c>
       <c r="I84" s="14" t="s">
-        <v>346</v>
-      </c>
-      <c r="J84" s="14"/>
+        <v>379</v>
+      </c>
+      <c r="J84" s="14" t="s">
+        <v>380</v>
+      </c>
       <c r="K84" s="16"/>
     </row>
     <row r="85" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4551,10 +4696,10 @@
         <v>12</v>
       </c>
       <c r="C85" s="14" t="s">
-        <v>347</v>
+        <v>372</v>
       </c>
       <c r="D85" s="15" t="s">
-        <v>348</v>
+        <v>381</v>
       </c>
       <c r="E85" s="13" t="s">
         <v>15</v>
@@ -4562,13 +4707,13 @@
       <c r="F85" s="13"/>
       <c r="G85" s="13"/>
       <c r="H85" s="14" t="s">
-        <v>349</v>
+        <v>382</v>
       </c>
       <c r="I85" s="14" t="s">
-        <v>350</v>
+        <v>383</v>
       </c>
       <c r="J85" s="14" t="s">
-        <v>351</v>
+        <v>384</v>
       </c>
       <c r="K85" s="16"/>
     </row>
@@ -4580,23 +4725,25 @@
         <v>12</v>
       </c>
       <c r="C86" s="14" t="s">
-        <v>347</v>
+        <v>372</v>
       </c>
       <c r="D86" s="15" t="s">
-        <v>352</v>
+        <v>385</v>
       </c>
       <c r="E86" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F86" s="13"/>
       <c r="G86" s="13"/>
       <c r="H86" s="14" t="s">
-        <v>353</v>
+        <v>386</v>
       </c>
       <c r="I86" s="14" t="s">
-        <v>354</v>
-      </c>
-      <c r="J86" s="14"/>
+        <v>387</v>
+      </c>
+      <c r="J86" s="14" t="s">
+        <v>388</v>
+      </c>
       <c r="K86" s="16"/>
     </row>
     <row r="87" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4607,23 +4754,25 @@
         <v>12</v>
       </c>
       <c r="C87" s="14" t="s">
-        <v>347</v>
+        <v>372</v>
       </c>
       <c r="D87" s="15" t="s">
-        <v>355</v>
+        <v>389</v>
       </c>
       <c r="E87" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F87" s="13"/>
       <c r="G87" s="13"/>
       <c r="H87" s="14" t="s">
-        <v>356</v>
+        <v>390</v>
       </c>
       <c r="I87" s="14" t="s">
-        <v>357</v>
-      </c>
-      <c r="J87" s="14"/>
+        <v>391</v>
+      </c>
+      <c r="J87" s="14" t="s">
+        <v>392</v>
+      </c>
       <c r="K87" s="16"/>
     </row>
     <row r="88" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4634,23 +4783,25 @@
         <v>12</v>
       </c>
       <c r="C88" s="14" t="s">
-        <v>347</v>
+        <v>393</v>
       </c>
       <c r="D88" s="15" t="s">
-        <v>358</v>
+        <v>394</v>
       </c>
       <c r="E88" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F88" s="13"/>
       <c r="G88" s="13"/>
       <c r="H88" s="14" t="s">
-        <v>359</v>
+        <v>395</v>
       </c>
       <c r="I88" s="14" t="s">
-        <v>360</v>
-      </c>
-      <c r="J88" s="14"/>
+        <v>396</v>
+      </c>
+      <c r="J88" s="14" t="s">
+        <v>397</v>
+      </c>
       <c r="K88" s="16"/>
     </row>
     <row r="89" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4661,23 +4812,25 @@
         <v>12</v>
       </c>
       <c r="C89" s="14" t="s">
-        <v>347</v>
+        <v>393</v>
       </c>
       <c r="D89" s="15" t="s">
-        <v>361</v>
+        <v>398</v>
       </c>
       <c r="E89" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F89" s="13"/>
       <c r="G89" s="13"/>
       <c r="H89" s="14" t="s">
-        <v>362</v>
+        <v>399</v>
       </c>
       <c r="I89" s="14" t="s">
-        <v>363</v>
-      </c>
-      <c r="J89" s="14"/>
+        <v>400</v>
+      </c>
+      <c r="J89" s="14" t="s">
+        <v>401</v>
+      </c>
       <c r="K89" s="16"/>
     </row>
     <row r="90" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4688,10 +4841,10 @@
         <v>12</v>
       </c>
       <c r="C90" s="14" t="s">
-        <v>364</v>
+        <v>393</v>
       </c>
       <c r="D90" s="15" t="s">
-        <v>365</v>
+        <v>402</v>
       </c>
       <c r="E90" s="13" t="s">
         <v>15</v>
@@ -4699,13 +4852,13 @@
       <c r="F90" s="13"/>
       <c r="G90" s="13"/>
       <c r="H90" s="14" t="s">
-        <v>366</v>
+        <v>403</v>
       </c>
       <c r="I90" s="14" t="s">
-        <v>367</v>
+        <v>404</v>
       </c>
       <c r="J90" s="14" t="s">
-        <v>368</v>
+        <v>405</v>
       </c>
       <c r="K90" s="16"/>
     </row>
@@ -4717,10 +4870,10 @@
         <v>12</v>
       </c>
       <c r="C91" s="14" t="s">
-        <v>364</v>
+        <v>393</v>
       </c>
       <c r="D91" s="15" t="s">
-        <v>369</v>
+        <v>406</v>
       </c>
       <c r="E91" s="13" t="s">
         <v>15</v>
@@ -4728,13 +4881,13 @@
       <c r="F91" s="13"/>
       <c r="G91" s="13"/>
       <c r="H91" s="14" t="s">
-        <v>370</v>
+        <v>407</v>
       </c>
       <c r="I91" s="14" t="s">
-        <v>371</v>
+        <v>408</v>
       </c>
       <c r="J91" s="14" t="s">
-        <v>372</v>
+        <v>409</v>
       </c>
       <c r="K91" s="16"/>
     </row>
@@ -4746,10 +4899,10 @@
         <v>12</v>
       </c>
       <c r="C92" s="14" t="s">
-        <v>364</v>
+        <v>393</v>
       </c>
       <c r="D92" s="15" t="s">
-        <v>373</v>
+        <v>410</v>
       </c>
       <c r="E92" s="13" t="s">
         <v>15</v>
@@ -4757,13 +4910,13 @@
       <c r="F92" s="13"/>
       <c r="G92" s="13"/>
       <c r="H92" s="14" t="s">
-        <v>374</v>
+        <v>411</v>
       </c>
       <c r="I92" s="14" t="s">
-        <v>375</v>
+        <v>412</v>
       </c>
       <c r="J92" s="14" t="s">
-        <v>376</v>
+        <v>413</v>
       </c>
       <c r="K92" s="16"/>
     </row>
@@ -4775,10 +4928,10 @@
         <v>12</v>
       </c>
       <c r="C93" s="14" t="s">
-        <v>364</v>
+        <v>393</v>
       </c>
       <c r="D93" s="15" t="s">
-        <v>377</v>
+        <v>414</v>
       </c>
       <c r="E93" s="13" t="s">
         <v>15</v>
@@ -4786,13 +4939,13 @@
       <c r="F93" s="13"/>
       <c r="G93" s="13"/>
       <c r="H93" s="14" t="s">
-        <v>378</v>
+        <v>415</v>
       </c>
       <c r="I93" s="14" t="s">
-        <v>379</v>
+        <v>416</v>
       </c>
       <c r="J93" s="14" t="s">
-        <v>380</v>
+        <v>417</v>
       </c>
       <c r="K93" s="16"/>
     </row>
@@ -4804,23 +4957,25 @@
         <v>12</v>
       </c>
       <c r="C94" s="14" t="s">
-        <v>364</v>
+        <v>393</v>
       </c>
       <c r="D94" s="15" t="s">
-        <v>381</v>
+        <v>418</v>
       </c>
       <c r="E94" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F94" s="13"/>
       <c r="G94" s="13"/>
       <c r="H94" s="14" t="s">
-        <v>382</v>
+        <v>419</v>
       </c>
       <c r="I94" s="14" t="s">
-        <v>383</v>
-      </c>
-      <c r="J94" s="14"/>
+        <v>420</v>
+      </c>
+      <c r="J94" s="14" t="s">
+        <v>421</v>
+      </c>
       <c r="K94" s="16"/>
     </row>
     <row r="95" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4831,23 +4986,25 @@
         <v>12</v>
       </c>
       <c r="C95" s="14" t="s">
-        <v>364</v>
+        <v>422</v>
       </c>
       <c r="D95" s="15" t="s">
-        <v>384</v>
+        <v>423</v>
       </c>
       <c r="E95" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F95" s="13"/>
       <c r="G95" s="13"/>
       <c r="H95" s="14" t="s">
-        <v>385</v>
+        <v>424</v>
       </c>
       <c r="I95" s="14" t="s">
-        <v>386</v>
-      </c>
-      <c r="J95" s="14"/>
+        <v>425</v>
+      </c>
+      <c r="J95" s="14" t="s">
+        <v>426</v>
+      </c>
       <c r="K95" s="16"/>
     </row>
     <row r="96" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4858,23 +5015,25 @@
         <v>12</v>
       </c>
       <c r="C96" s="14" t="s">
-        <v>364</v>
+        <v>422</v>
       </c>
       <c r="D96" s="15" t="s">
-        <v>387</v>
+        <v>427</v>
       </c>
       <c r="E96" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F96" s="13"/>
       <c r="G96" s="13"/>
       <c r="H96" s="14" t="s">
-        <v>388</v>
+        <v>428</v>
       </c>
       <c r="I96" s="14" t="s">
-        <v>389</v>
-      </c>
-      <c r="J96" s="14"/>
+        <v>429</v>
+      </c>
+      <c r="J96" s="14" t="s">
+        <v>430</v>
+      </c>
       <c r="K96" s="16"/>
     </row>
     <row r="97" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4885,99 +5044,43 @@
         <v>12</v>
       </c>
       <c r="C97" s="14" t="s">
-        <v>390</v>
+        <v>422</v>
       </c>
       <c r="D97" s="15" t="s">
-        <v>391</v>
+        <v>431</v>
       </c>
       <c r="E97" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F97" s="13"/>
       <c r="G97" s="13"/>
       <c r="H97" s="14" t="s">
-        <v>392</v>
+        <v>432</v>
       </c>
       <c r="I97" s="14" t="s">
-        <v>393</v>
-      </c>
-      <c r="J97" s="14"/>
+        <v>433</v>
+      </c>
+      <c r="J97" s="14" t="s">
+        <v>434</v>
+      </c>
       <c r="K97" s="16"/>
     </row>
-    <row r="98" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="13" t="n">
-        <v>97</v>
-      </c>
-      <c r="B98" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="C98" s="14" t="s">
-        <v>390</v>
-      </c>
-      <c r="D98" s="15" t="s">
-        <v>394</v>
-      </c>
-      <c r="E98" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F98" s="13"/>
-      <c r="G98" s="13"/>
-      <c r="H98" s="14" t="s">
-        <v>395</v>
-      </c>
-      <c r="I98" s="14" t="s">
-        <v>396</v>
-      </c>
-      <c r="J98" s="14" t="s">
-        <v>397</v>
-      </c>
-      <c r="K98" s="16"/>
-    </row>
-    <row r="99" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="13" t="n">
-        <v>98</v>
-      </c>
-      <c r="B99" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="C99" s="14" t="s">
-        <v>390</v>
-      </c>
-      <c r="D99" s="15" t="s">
-        <v>398</v>
-      </c>
-      <c r="E99" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="F99" s="13"/>
-      <c r="G99" s="13"/>
-      <c r="H99" s="14" t="s">
-        <v>399</v>
-      </c>
-      <c r="I99" s="14" t="s">
-        <v>400</v>
-      </c>
-      <c r="J99" s="14" t="s">
-        <v>401</v>
-      </c>
-      <c r="K99" s="16"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K99"/>
-  <conditionalFormatting sqref="E2:E99">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+  <autoFilter ref="A1:K97"/>
+  <conditionalFormatting sqref="E2:E97">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>"Ada"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>"Belum"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E99" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E2:E97" type="list">
       <formula1>"Ada,Belum,Sebagian"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K2:K99" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K2:K97" type="list">
       <formula1>"P1 - Quick win,P2 - Pembeda,P3 - Naik kelas,P4 - Skala"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -5007,42 +5110,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
-        <v>402</v>
+        <v>435</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>404</v>
+        <v>437</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
-        <v>406</v>
+        <v>439</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>407</v>
+        <v>440</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>408</v>
+        <v>441</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>410</v>
+        <v>443</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>411</v>
+        <v>444</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
WhatsApp: pakai library Api_Whatsapp milik sendiri (wa_notif) untuk semua notifikasi
- Api_Whatsapp di-autoload hanya bila application/libraries/Api_Whatsapp.php
  ada (berkasnya di .gitignore), supaya salinan repo tanpa berkas itu tetap jalan.
- Notifikasi_lib::wa() memanggil $this->api_whatsapp->wa_notif($pesan, $nomor)
  bila tersedia; gerbang format Fonnte jadi cadangan. Galat dari gerbang
  dicatat sebagai 'gagal' dan tidak menggagalkan proses yang memicunya.
- Saklar 'Kirim notifikasi WhatsApp' aktif bawaan bila Api_Whatsapp terpasang.
- Dokumen rancangan & lembar QA diperbarui.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HmiNd1QbTyjAfj7oGbYGxq
</commit_message>
<xml_diff>
--- a/docs/rancangan-fitur-marketplace-umkm.xlsx
+++ b/docs/rancangan-fitur-marketplace-umkm.xlsx
@@ -238,7 +238,7 @@
     <t xml:space="preserve">3. config/surat.php berisi SMTP uji (mis. Mailtrap) supaya email tidak sampai ke pengguna sungguhan.</t>
   </si>
   <si>
-    <t xml:space="preserve">4. Gerbang WhatsApp memakai nomor uji; kunci agregator ekspedisi mode uji (Admin &gt; Pengaturan).</t>
+    <t xml:space="preserve">4. Api_Whatsapp.php terpasang dan mengirim ke nomor uji; kunci agregator ekspedisi mode uji (Admin &gt; Pengaturan).</t>
   </si>
   <si>
     <t xml:space="preserve">5. Akun uji: 1 admin, 1 pendamping, 2 penjual (toko di 2 kota berbeda), 2 pembeli, + uji sebagai tamu.</t>
@@ -688,7 +688,7 @@
     <t xml:space="preserve">Kabar status pesanan dikirim ke WA.</t>
   </si>
   <si>
-    <t xml:space="preserve">Notifikasi_lib — WA (format Fonnte) &amp; email; aktifkan di Admin &gt; Pengaturan.</t>
+    <t xml:space="preserve">Notifikasi_lib — WA lewat library Api_Whatsapp milik sendiri (wa_notif), cadangan gerbang format Fonnte; email lewat SMTP. Saklar di Admin &gt; Pengaturan.</t>
   </si>
   <si>
     <t xml:space="preserve">Pengalaman &amp; Aksesibilitas</t>
@@ -1507,7 +1507,7 @@
     <t xml:space="preserve">Langkah 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Salin application/config/surat.example.php menjadi surat.php dan isi SMTP (dipakai email reset sandi, verifikasi, dan notifikasi). Isi kunci di Admin &gt; Pengaturan: gerbang WhatsApp (mis. Fonnte) dan agregator ekspedisi (mis. Biteship). Tanpa kunci, fitur tetap jalan dengan cara manual (tautan WA, tautan lacak resmi kurir).</t>
+    <t xml:space="preserve">Salin application/config/surat.example.php menjadi surat.php dan isi SMTP (dipakai email reset sandi, verifikasi, dan notifikasi). Taruh application/libraries/Api_Whatsapp.php (gerbang WA sendiri, tidak ikut di repo) - otomatis di-autoload dan dipakai semua notifikasi WA. Isi kunci agregator ekspedisi (mis. Biteship) di Admin &gt; Pengaturan. Tanpa kunci, fitur tetap jalan dengan cara manual (tautan WA, tautan lacak resmi kurir).</t>
   </si>
   <si>
     <t xml:space="preserve">Langkah 3</t>
@@ -1683,7 +1683,7 @@
     <t xml:space="preserve">Masuk dengan kode OTP</t>
   </si>
   <si>
-    <t xml:space="preserve">Gerbang WA aktif (Admin &gt; Pengaturan); akun punya nomor WA unik</t>
+    <t xml:space="preserve">Api_Whatsapp.php terpasang &amp; WA aktif di Admin &gt; Pengaturan; akun punya nomor WA unik</t>
   </si>
   <si>
     <t xml:space="preserve">1. Buka /auth/otp
@@ -1777,7 +1777,7 @@
     <t xml:space="preserve">Reset sandi lewat nomor WhatsApp</t>
   </si>
   <si>
-    <t xml:space="preserve">Gerbang WA aktif</t>
+    <t xml:space="preserve">Api_Whatsapp.php terpasang &amp; WA aktif di Admin &gt; Pengaturan</t>
   </si>
   <si>
     <t xml:space="preserve">1. Buka /auth/lupa
@@ -2451,16 +2451,16 @@
     <t xml:space="preserve">TC-PBL-054</t>
   </si>
   <si>
-    <t xml:space="preserve">Gerbang WA mati / token salah</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Token WA salah</t>
+    <t xml:space="preserve">Gerbang WA error / tidak terhubung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Api_Whatsapp gagal (mis. layanan WA dimatikan sementara)</t>
   </si>
   <si>
     <t xml:space="preserve">1. Bayar pesanan</t>
   </si>
   <si>
-    <t xml:space="preserve">Pesanan tetap diproses normal; log notifikasi berstatus gagal, tidak ada halaman galat.</t>
+    <t xml:space="preserve">Pesanan tetap Lunas &amp; diproses normal; di Admin &gt; Pengaturan &gt; Notifikasi tercatat "gagal" beserta pesan galatnya; tidak ada halaman galat.</t>
   </si>
   <si>
     <t xml:space="preserve">TC-PBL-055</t>
@@ -6636,7 +6636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="19" t="n">
         <v>33</v>
       </c>
@@ -9144,7 +9144,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
         <v>491</v>
       </c>
@@ -11584,7 +11584,7 @@
       <c r="O54" s="26"/>
       <c r="P54" s="25"/>
     </row>
-    <row r="55" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="19" t="s">
         <v>784</v>
       </c>

</xml_diff>

<commit_message>
Api_Whatsapp: aman dipakai tanpa tabel utility, keluaran PHP gerbang tidak bocor ke halaman
- Migrasi 33: tabel utility (server_wa = bind/fast_wa/kirimi) yang dibaca
  Api_Whatsapp; tabel yang sudah ada tidak diubah selain menambah kolom.
- Notifikasi_lib::wa(): cek tabel utility dulu (tanpa itu db_debug
  menghentikan checkout/callback), bungkus keluaran gerbang supaya peringatan
  PHP tidak merusak balasan JSON, baca balasan success/status=false bila
  wa_notif() kelak mengembalikan nilai.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HmiNd1QbTyjAfj7oGbYGxq
</commit_message>
<xml_diff>
--- a/docs/rancangan-fitur-marketplace-umkm.xlsx
+++ b/docs/rancangan-fitur-marketplace-umkm.xlsx
@@ -229,7 +229,7 @@
     <t xml:space="preserve">Lingkungan Uji (siapkan sebelum mulai)</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Server staging terpisah dari produksi, database hasil migrasi database/15 s.d. 32 (cadangkan dulu).</t>
+    <t xml:space="preserve">1. Server staging terpisah dari produksi, database hasil migrasi database/15 s.d. 33 (cadangkan dulu).</t>
   </si>
   <si>
     <t xml:space="preserve">2. Duitku mode SANDBOX (jangan memakai kunci produksi saat menguji pembayaran).</t>
@@ -1501,13 +1501,13 @@
     <t xml:space="preserve">Langkah 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Jalankan migrasi database/24_*.sql sampai database/32_*.sql berurutan (aman diulang; cadangkan dulu). Urutan penting: 26_pengaturan_notifikasi.sql menambah kolom ke tabel auth_tokens dari 25_reset_sandi_verifikasi.sql.</t>
+    <t xml:space="preserve">Jalankan migrasi database/24_*.sql sampai database/33_*.sql berurutan (aman diulang; cadangkan dulu). Urutan penting: 26_pengaturan_notifikasi.sql menambah kolom ke tabel auth_tokens dari 25_reset_sandi_verifikasi.sql.</t>
   </si>
   <si>
     <t xml:space="preserve">Langkah 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Salin application/config/surat.example.php menjadi surat.php dan isi SMTP (dipakai email reset sandi, verifikasi, dan notifikasi). Taruh application/libraries/Api_Whatsapp.php (gerbang WA sendiri, tidak ikut di repo) - otomatis di-autoload dan dipakai semua notifikasi WA. Isi kunci agregator ekspedisi (mis. Biteship) di Admin &gt; Pengaturan. Tanpa kunci, fitur tetap jalan dengan cara manual (tautan WA, tautan lacak resmi kurir).</t>
+    <t xml:space="preserve">Salin application/config/surat.example.php menjadi surat.php dan isi SMTP (dipakai email reset sandi, verifikasi, dan notifikasi). Taruh application/libraries/Api_Whatsapp.php (gerbang WA sendiri, tidak ikut di repo) - otomatis di-autoload dan dipakai semua notifikasi WA; server WA dipilih lewat utility.server_wa (bind / fast_wa / kirimi, tabel dibuat 33_utility_wa.sql). Isi kunci agregator ekspedisi (mis. Biteship) di Admin &gt; Pengaturan. Tanpa kunci, fitur tetap jalan dengan cara manual (tautan WA, tautan lacak resmi kurir).</t>
   </si>
   <si>
     <t xml:space="preserve">Langkah 3</t>
@@ -9144,7 +9144,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="21" t="s">
         <v>491</v>
       </c>

</xml_diff>

<commit_message>
Hapus migrasi 33_utility_wa: tabel utility (pilihan server WA) sudah ada di database pemilik
Pengecekan tabel utility di Notifikasi_lib tetap ada sebagai pengaman.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HmiNd1QbTyjAfj7oGbYGxq
</commit_message>
<xml_diff>
--- a/docs/rancangan-fitur-marketplace-umkm.xlsx
+++ b/docs/rancangan-fitur-marketplace-umkm.xlsx
@@ -229,7 +229,7 @@
     <t xml:space="preserve">Lingkungan Uji (siapkan sebelum mulai)</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Server staging terpisah dari produksi, database hasil migrasi database/15 s.d. 33 (cadangkan dulu).</t>
+    <t xml:space="preserve">1. Server staging terpisah dari produksi, database hasil migrasi database/15 s.d. 32 (cadangkan dulu).</t>
   </si>
   <si>
     <t xml:space="preserve">2. Duitku mode SANDBOX (jangan memakai kunci produksi saat menguji pembayaran).</t>
@@ -1501,13 +1501,13 @@
     <t xml:space="preserve">Langkah 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Jalankan migrasi database/24_*.sql sampai database/33_*.sql berurutan (aman diulang; cadangkan dulu). Urutan penting: 26_pengaturan_notifikasi.sql menambah kolom ke tabel auth_tokens dari 25_reset_sandi_verifikasi.sql.</t>
+    <t xml:space="preserve">Jalankan migrasi database/24_*.sql sampai database/32_*.sql berurutan (aman diulang; cadangkan dulu). Urutan penting: 26_pengaturan_notifikasi.sql menambah kolom ke tabel auth_tokens dari 25_reset_sandi_verifikasi.sql.</t>
   </si>
   <si>
     <t xml:space="preserve">Langkah 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Salin application/config/surat.example.php menjadi surat.php dan isi SMTP (dipakai email reset sandi, verifikasi, dan notifikasi). Taruh application/libraries/Api_Whatsapp.php (gerbang WA sendiri, tidak ikut di repo) - otomatis di-autoload dan dipakai semua notifikasi WA; server WA dipilih lewat utility.server_wa (bind / fast_wa / kirimi, tabel dibuat 33_utility_wa.sql). Isi kunci agregator ekspedisi (mis. Biteship) di Admin &gt; Pengaturan. Tanpa kunci, fitur tetap jalan dengan cara manual (tautan WA, tautan lacak resmi kurir).</t>
+    <t xml:space="preserve">Salin application/config/surat.example.php menjadi surat.php dan isi SMTP (dipakai email reset sandi, verifikasi, dan notifikasi). Taruh application/libraries/Api_Whatsapp.php (gerbang WA sendiri, tidak ikut di repo) - otomatis di-autoload dan dipakai semua notifikasi WA; server WA dipilih lewat utility.server_wa (bind / fast_wa / kirimi) di database Anda. Isi kunci agregator ekspedisi (mis. Biteship) di Admin &gt; Pengaturan. Tanpa kunci, fitur tetap jalan dengan cara manual (tautan WA, tautan lacak resmi kurir).</t>
   </si>
   <si>
     <t xml:space="preserve">Langkah 3</t>

</xml_diff>

<commit_message>
Data wilayah lengkap: 38 provinsi, 514 kab/kota, 7.285 kecamatan (Kepmendagri 2025)
- Migrasi 33_wilayah_indonesia.sql (sumber: cahyadsn/wilayah, MIT).
  Wilayah yang sudah ada dicocokkan lewat nama (atau kode untuk yang
  berganti nama, atau nama nasional untuk pemekaran Papua) sehingga ID-nya
  tetap dan toko/alamat/pesanan tidak putus; sisanya ditambahkan. Aman
  dijalankan berulang, tanpa duplikat, untuk data berformat Kemendagri
  maupun BPS.
- Region_model: pencocokan peta mengenali nama Jakarta/Yogyakarta/Aceh
  versi lama/baru dan nama yang hanya beda spasi (Pal Merah vs Palmerah).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HmiNd1QbTyjAfj7oGbYGxq
</commit_message>
<xml_diff>
--- a/docs/rancangan-fitur-marketplace-umkm.xlsx
+++ b/docs/rancangan-fitur-marketplace-umkm.xlsx
@@ -229,7 +229,7 @@
     <t xml:space="preserve">Lingkungan Uji (siapkan sebelum mulai)</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Server staging terpisah dari produksi, database hasil migrasi database/15 s.d. 32 (cadangkan dulu).</t>
+    <t xml:space="preserve">1. Server staging terpisah dari produksi, database hasil migrasi database/15 s.d. 33 (cadangkan dulu).</t>
   </si>
   <si>
     <t xml:space="preserve">2. Duitku mode SANDBOX (jangan memakai kunci produksi saat menguji pembayaran).</t>
@@ -1501,7 +1501,7 @@
     <t xml:space="preserve">Langkah 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Jalankan migrasi database/24_*.sql sampai database/32_*.sql berurutan (aman diulang; cadangkan dulu). Urutan penting: 26_pengaturan_notifikasi.sql menambah kolom ke tabel auth_tokens dari 25_reset_sandi_verifikasi.sql.</t>
+    <t xml:space="preserve">Jalankan migrasi database/24_*.sql sampai database/33_*.sql berurutan (aman diulang; cadangkan dulu). 33_wilayah_indonesia.sql mengisi data wilayah lengkap (38 provinsi, 514 kab/kota, 7.285 kecamatan, Kepmendagri 2025) tanpa mengubah ID wilayah yang sudah dipakai. Urutan penting: 26_pengaturan_notifikasi.sql menambah kolom ke tabel auth_tokens dari 25_reset_sandi_verifikasi.sql.</t>
   </si>
   <si>
     <t xml:space="preserve">Langkah 2</t>
@@ -9136,7 +9136,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="21" t="s">
         <v>489</v>
       </c>

</xml_diff>

<commit_message>
Chat: pesan pembeli dari halaman pesanan kini sampai ke kotak masuk penjual
- Chat_model::kirim() menyimpan pesan ke wadah percakapan pesanan
  (conversation_id), bukan hanya order_id. Sebelumnya pesan pembeli dari
  halaman pesanan dan catatan sistem tidak muncul di menu Pesan penjual,
  yang membaca lewat conversation_id.
- Lencana 'Pesan' di panel penjual menghitung semua percakapan toko,
  termasuk 'tanya sebelum beli' (belum_dibaca_toko_total); sebelumnya
  pertanyaan calon pembeli tidak pernah menyalakan lencana.
- Migrasi 34_chat_percakapan.sql menautkan pesan lama yang belum punya
  percakapan. Tidak ada pesan yang dihapus.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HmiNd1QbTyjAfj7oGbYGxq
</commit_message>
<xml_diff>
--- a/docs/rancangan-fitur-marketplace-umkm.xlsx
+++ b/docs/rancangan-fitur-marketplace-umkm.xlsx
@@ -229,7 +229,7 @@
     <t xml:space="preserve">Lingkungan Uji (siapkan sebelum mulai)</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Server staging terpisah dari produksi, database hasil migrasi database/15 s.d. 33 (cadangkan dulu).</t>
+    <t xml:space="preserve">1. Server staging terpisah dari produksi, database hasil migrasi database/15 s.d. 34 (cadangkan dulu).</t>
   </si>
   <si>
     <t xml:space="preserve">2. Duitku mode SANDBOX (jangan memakai kunci produksi saat menguji pembayaran).</t>
@@ -1501,7 +1501,7 @@
     <t xml:space="preserve">Langkah 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Jalankan migrasi database/24_*.sql sampai database/33_*.sql berurutan (aman diulang; cadangkan dulu). 33_wilayah_indonesia.sql mengisi data wilayah lengkap (38 provinsi, 514 kab/kota, 7.285 kecamatan, Kepmendagri 2025) tanpa mengubah ID wilayah yang sudah dipakai. Urutan penting: 26_pengaturan_notifikasi.sql menambah kolom ke tabel auth_tokens dari 25_reset_sandi_verifikasi.sql.</t>
+    <t xml:space="preserve">Jalankan migrasi database/24_*.sql sampai database/34_*.sql berurutan (aman diulang; cadangkan dulu). 33_wilayah_indonesia.sql mengisi data wilayah lengkap (38 provinsi, 514 kab/kota, 7.285 kecamatan, Kepmendagri 2025) tanpa mengubah ID wilayah yang sudah dipakai. Urutan penting: 26_pengaturan_notifikasi.sql menambah kolom ke tabel auth_tokens dari 25_reset_sandi_verifikasi.sql.</t>
   </si>
   <si>
     <t xml:space="preserve">Langkah 2</t>

</xml_diff>